<commit_message>
Įvestas Skaiciavimai.py sustabdymas pradiniu duomenu ivedimui ir nuskaitymui
</commit_message>
<xml_diff>
--- a/Ivestis1.xlsx
+++ b/Ivestis1.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="263" documentId="13_ncr:1_{D8ED3FA4-1188-4E70-924F-660A50F19C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8685D0F3-FD86-4775-8711-4CB6F11BBCB9}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="3" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="1" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Compatibility Report" sheetId="4" state="hidden" r:id="rId1"/>
@@ -2668,200 +2668,200 @@
     <xf numFmtId="164" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="30" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="30" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -3293,31 +3293,31 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="D2" s="246" t="s">
+      <c r="D2" s="245" t="s">
         <v>108</v>
       </c>
-      <c r="E2" s="246"/>
-      <c r="F2" s="246"/>
-      <c r="G2" s="246"/>
-      <c r="H2" s="246"/>
-      <c r="I2" s="246"/>
-      <c r="J2" s="246"/>
-      <c r="K2" s="246"/>
-      <c r="L2" s="246"/>
-      <c r="M2" s="246"/>
-      <c r="N2" s="246"/>
-      <c r="O2" s="246"/>
-      <c r="P2" s="246"/>
-      <c r="Q2" s="246"/>
-      <c r="R2" s="246"/>
-      <c r="S2" s="246"/>
-      <c r="T2" s="246"/>
-      <c r="U2" s="246"/>
-      <c r="V2" s="246"/>
-      <c r="W2" s="246"/>
-      <c r="X2" s="246"/>
-      <c r="Y2" s="246"/>
-      <c r="Z2" s="246"/>
+      <c r="E2" s="245"/>
+      <c r="F2" s="245"/>
+      <c r="G2" s="245"/>
+      <c r="H2" s="245"/>
+      <c r="I2" s="245"/>
+      <c r="J2" s="245"/>
+      <c r="K2" s="245"/>
+      <c r="L2" s="245"/>
+      <c r="M2" s="245"/>
+      <c r="N2" s="245"/>
+      <c r="O2" s="245"/>
+      <c r="P2" s="245"/>
+      <c r="Q2" s="245"/>
+      <c r="R2" s="245"/>
+      <c r="S2" s="245"/>
+      <c r="T2" s="245"/>
+      <c r="U2" s="245"/>
+      <c r="V2" s="245"/>
+      <c r="W2" s="245"/>
+      <c r="X2" s="245"/>
+      <c r="Y2" s="245"/>
+      <c r="Z2" s="245"/>
     </row>
     <row r="4" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
@@ -3406,13 +3406,13 @@
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A5" s="247">
+      <c r="A5" s="246">
         <v>46063</v>
       </c>
-      <c r="B5" s="250">
+      <c r="B5" s="249">
         <v>5</v>
       </c>
-      <c r="C5" s="253" t="s">
+      <c r="C5" s="252" t="s">
         <v>140</v>
       </c>
       <c r="D5" s="177">
@@ -3503,14 +3503,14 @@
         <f>Aerodinamika!G27</f>
         <v>1.3179692000000001</v>
       </c>
-      <c r="AB5" s="244" t="s">
+      <c r="AB5" s="243" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A6" s="248"/>
-      <c r="B6" s="251"/>
-      <c r="C6" s="254"/>
+      <c r="A6" s="247"/>
+      <c r="B6" s="250"/>
+      <c r="C6" s="253"/>
       <c r="D6" s="177">
         <v>16</v>
       </c>
@@ -3595,12 +3595,12 @@
         <f>O5*X6</f>
         <v>0.79775867584824989</v>
       </c>
-      <c r="AB6" s="245"/>
+      <c r="AB6" s="244"/>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="248"/>
-      <c r="B7" s="251"/>
-      <c r="C7" s="254"/>
+      <c r="A7" s="247"/>
+      <c r="B7" s="250"/>
+      <c r="C7" s="253"/>
       <c r="D7" s="200">
         <v>31</v>
       </c>
@@ -3651,9 +3651,9 @@
       <c r="S7" s="176"/>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="248"/>
-      <c r="B8" s="251"/>
-      <c r="C8" s="254"/>
+      <c r="A8" s="247"/>
+      <c r="B8" s="250"/>
+      <c r="C8" s="253"/>
       <c r="D8" s="177">
         <v>60</v>
       </c>
@@ -3708,9 +3708,9 @@
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A9" s="248"/>
-      <c r="B9" s="251"/>
-      <c r="C9" s="254"/>
+      <c r="A9" s="247"/>
+      <c r="B9" s="250"/>
+      <c r="C9" s="253"/>
       <c r="D9" s="177">
         <v>89</v>
       </c>
@@ -3754,9 +3754,9 @@
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A10" s="248"/>
-      <c r="B10" s="251"/>
-      <c r="C10" s="254"/>
+      <c r="A10" s="247"/>
+      <c r="B10" s="250"/>
+      <c r="C10" s="253"/>
       <c r="D10" s="177">
         <v>104</v>
       </c>
@@ -3800,9 +3800,9 @@
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A11" s="249"/>
-      <c r="B11" s="252"/>
-      <c r="C11" s="255"/>
+      <c r="A11" s="248"/>
+      <c r="B11" s="251"/>
+      <c r="C11" s="254"/>
       <c r="D11" s="177">
         <v>115</v>
       </c>
@@ -3871,18 +3871,18 @@
       <c r="D13" s="200" t="s">
         <v>135</v>
       </c>
-      <c r="E13" s="256" t="s">
+      <c r="E13" s="255" t="s">
         <v>136</v>
       </c>
-      <c r="F13" s="257"/>
-      <c r="G13" s="257"/>
-      <c r="H13" s="257"/>
-      <c r="I13" s="257"/>
-      <c r="J13" s="257"/>
-      <c r="K13" s="257"/>
-      <c r="L13" s="257"/>
-      <c r="M13" s="257"/>
-      <c r="N13" s="258"/>
+      <c r="F13" s="256"/>
+      <c r="G13" s="256"/>
+      <c r="H13" s="256"/>
+      <c r="I13" s="256"/>
+      <c r="J13" s="256"/>
+      <c r="K13" s="256"/>
+      <c r="L13" s="256"/>
+      <c r="M13" s="256"/>
+      <c r="N13" s="257"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" s="206"/>
@@ -3917,31 +3917,31 @@
       <c r="A17" s="206"/>
       <c r="B17" s="206"/>
       <c r="C17" s="206"/>
-      <c r="D17" s="259" t="s">
+      <c r="D17" s="258" t="s">
         <v>138</v>
       </c>
-      <c r="E17" s="246"/>
-      <c r="F17" s="246"/>
-      <c r="G17" s="246"/>
-      <c r="H17" s="246"/>
-      <c r="I17" s="246"/>
-      <c r="J17" s="246"/>
-      <c r="K17" s="246"/>
-      <c r="L17" s="246"/>
-      <c r="M17" s="246"/>
-      <c r="N17" s="246"/>
-      <c r="O17" s="246"/>
-      <c r="P17" s="246"/>
-      <c r="Q17" s="246"/>
-      <c r="R17" s="246"/>
-      <c r="S17" s="246"/>
-      <c r="T17" s="246"/>
-      <c r="U17" s="246"/>
-      <c r="V17" s="246"/>
-      <c r="W17" s="246"/>
-      <c r="X17" s="246"/>
-      <c r="Y17" s="246"/>
-      <c r="Z17" s="246"/>
+      <c r="E17" s="245"/>
+      <c r="F17" s="245"/>
+      <c r="G17" s="245"/>
+      <c r="H17" s="245"/>
+      <c r="I17" s="245"/>
+      <c r="J17" s="245"/>
+      <c r="K17" s="245"/>
+      <c r="L17" s="245"/>
+      <c r="M17" s="245"/>
+      <c r="N17" s="245"/>
+      <c r="O17" s="245"/>
+      <c r="P17" s="245"/>
+      <c r="Q17" s="245"/>
+      <c r="R17" s="245"/>
+      <c r="S17" s="245"/>
+      <c r="T17" s="245"/>
+      <c r="U17" s="245"/>
+      <c r="V17" s="245"/>
+      <c r="W17" s="245"/>
+      <c r="X17" s="245"/>
+      <c r="Y17" s="245"/>
+      <c r="Z17" s="245"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" s="206"/>
@@ -4047,9 +4047,9 @@
       </c>
     </row>
     <row r="20" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="260"/>
-      <c r="B20" s="260"/>
-      <c r="C20" s="260"/>
+      <c r="A20" s="259"/>
+      <c r="B20" s="259"/>
+      <c r="C20" s="259"/>
       <c r="D20" s="177">
         <v>3</v>
       </c>
@@ -4126,12 +4126,12 @@
       <c r="AA20" s="219">
         <v>1.35</v>
       </c>
-      <c r="AB20" s="244"/>
+      <c r="AB20" s="243"/>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A21" s="261"/>
-      <c r="B21" s="261"/>
-      <c r="C21" s="261"/>
+      <c r="A21" s="260"/>
+      <c r="B21" s="260"/>
+      <c r="C21" s="260"/>
       <c r="D21" s="177">
         <v>15</v>
       </c>
@@ -4202,12 +4202,12 @@
         <f>O20*X21</f>
         <v>1.0671545706141219</v>
       </c>
-      <c r="AB21" s="245"/>
+      <c r="AB21" s="244"/>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A22" s="261"/>
-      <c r="B22" s="261"/>
-      <c r="C22" s="261"/>
+      <c r="A22" s="260"/>
+      <c r="B22" s="260"/>
+      <c r="C22" s="260"/>
       <c r="D22" s="200">
         <v>27</v>
       </c>
@@ -4246,9 +4246,9 @@
       <c r="S22" s="176"/>
     </row>
     <row r="23" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A23" s="261"/>
-      <c r="B23" s="261"/>
-      <c r="C23" s="261"/>
+      <c r="A23" s="260"/>
+      <c r="B23" s="260"/>
+      <c r="C23" s="260"/>
       <c r="D23" s="177">
         <v>4</v>
       </c>
@@ -4291,9 +4291,9 @@
       </c>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A24" s="261"/>
-      <c r="B24" s="261"/>
-      <c r="C24" s="261"/>
+      <c r="A24" s="260"/>
+      <c r="B24" s="260"/>
+      <c r="C24" s="260"/>
       <c r="D24" s="177">
         <v>5</v>
       </c>
@@ -4325,9 +4325,9 @@
       </c>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A25" s="261"/>
-      <c r="B25" s="261"/>
-      <c r="C25" s="261"/>
+      <c r="A25" s="260"/>
+      <c r="B25" s="260"/>
+      <c r="C25" s="260"/>
       <c r="D25" s="177">
         <v>6</v>
       </c>
@@ -4359,9 +4359,9 @@
       </c>
     </row>
     <row r="26" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A26" s="262"/>
-      <c r="B26" s="262"/>
-      <c r="C26" s="262"/>
+      <c r="A26" s="261"/>
+      <c r="B26" s="261"/>
+      <c r="C26" s="261"/>
       <c r="D26" s="177">
         <v>7</v>
       </c>
@@ -4451,18 +4451,18 @@
       <c r="I2" s="10"/>
     </row>
     <row r="3" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="263" t="s">
+      <c r="A3" s="262" t="s">
         <v>107</v>
       </c>
-      <c r="B3" s="263"/>
-      <c r="C3" s="263"/>
-      <c r="D3" s="263"/>
-      <c r="E3" s="263"/>
-      <c r="F3" s="263"/>
-      <c r="G3" s="263"/>
-      <c r="H3" s="263"/>
-      <c r="I3" s="263"/>
-      <c r="J3" s="263"/>
+      <c r="B3" s="262"/>
+      <c r="C3" s="262"/>
+      <c r="D3" s="262"/>
+      <c r="E3" s="262"/>
+      <c r="F3" s="262"/>
+      <c r="G3" s="262"/>
+      <c r="H3" s="262"/>
+      <c r="I3" s="262"/>
+      <c r="J3" s="262"/>
     </row>
     <row r="4" spans="1:12" ht="14" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
@@ -4609,46 +4609,46 @@
       <c r="L10" s="45"/>
     </row>
     <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H11" s="264" t="s">
+      <c r="H11" s="263" t="s">
         <v>26</v>
       </c>
-      <c r="I11" s="267" t="s">
+      <c r="I11" s="266" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H12" s="265"/>
-      <c r="I12" s="268"/>
+      <c r="H12" s="264"/>
+      <c r="I12" s="267"/>
     </row>
     <row r="13" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H13" s="265"/>
-      <c r="I13" s="268"/>
+      <c r="H13" s="264"/>
+      <c r="I13" s="267"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H14" s="265"/>
-      <c r="I14" s="268"/>
+      <c r="H14" s="264"/>
+      <c r="I14" s="267"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H15" s="265"/>
-      <c r="I15" s="268"/>
+      <c r="H15" s="264"/>
+      <c r="I15" s="267"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H16" s="265"/>
-      <c r="I16" s="268"/>
+      <c r="H16" s="264"/>
+      <c r="I16" s="267"/>
     </row>
     <row r="17" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H17" s="265"/>
-      <c r="I17" s="268"/>
+      <c r="H17" s="264"/>
+      <c r="I17" s="267"/>
     </row>
     <row r="18" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H18" s="266"/>
-      <c r="I18" s="268"/>
+      <c r="H18" s="265"/>
+      <c r="I18" s="267"/>
     </row>
     <row r="19" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I19" s="268"/>
+      <c r="I19" s="267"/>
     </row>
     <row r="20" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I20" s="269"/>
+      <c r="I20" s="268"/>
     </row>
     <row r="21" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I21" s="57"/>
@@ -4710,35 +4710,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="275" t="s">
+      <c r="C1" s="274" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="275"/>
+      <c r="D1" s="274"/>
       <c r="E1" s="15"/>
       <c r="S1" s="16"/>
     </row>
     <row r="2" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="276" t="s">
+      <c r="A2" s="275" t="s">
         <v>97</v>
       </c>
-      <c r="B2" s="276"/>
-      <c r="C2" s="276"/>
-      <c r="D2" s="276"/>
-      <c r="E2" s="276"/>
-      <c r="F2" s="276"/>
-      <c r="G2" s="276"/>
-      <c r="H2" s="276"/>
-      <c r="I2" s="276"/>
-      <c r="J2" s="276"/>
-      <c r="K2" s="276"/>
-      <c r="L2" s="276"/>
-      <c r="M2" s="276"/>
-      <c r="N2" s="276"/>
-      <c r="O2" s="276"/>
-      <c r="P2" s="276"/>
-      <c r="Q2" s="276"/>
-      <c r="R2" s="276"/>
-      <c r="S2" s="276"/>
+      <c r="B2" s="275"/>
+      <c r="C2" s="275"/>
+      <c r="D2" s="275"/>
+      <c r="E2" s="275"/>
+      <c r="F2" s="275"/>
+      <c r="G2" s="275"/>
+      <c r="H2" s="275"/>
+      <c r="I2" s="275"/>
+      <c r="J2" s="275"/>
+      <c r="K2" s="275"/>
+      <c r="L2" s="275"/>
+      <c r="M2" s="275"/>
+      <c r="N2" s="275"/>
+      <c r="O2" s="275"/>
+      <c r="P2" s="275"/>
+      <c r="Q2" s="275"/>
+      <c r="R2" s="275"/>
+      <c r="S2" s="275"/>
     </row>
     <row r="3" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
@@ -4840,7 +4840,7 @@
       <c r="B6" s="229" t="s">
         <v>141</v>
       </c>
-      <c r="C6" s="271" t="str">
+      <c r="C6" s="270" t="str">
         <f>Greitis!C5</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -4912,7 +4912,7 @@
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="225"/>
       <c r="B7" s="226"/>
-      <c r="C7" s="272"/>
+      <c r="C7" s="271"/>
       <c r="D7" s="19"/>
       <c r="E7" s="20"/>
       <c r="F7" s="78">
@@ -4975,7 +4975,7 @@
     <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="225"/>
       <c r="B8" s="226"/>
-      <c r="C8" s="272"/>
+      <c r="C8" s="271"/>
       <c r="D8" s="19"/>
       <c r="E8" s="20"/>
       <c r="F8" s="78">
@@ -5038,7 +5038,7 @@
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="227"/>
       <c r="B9" s="227"/>
-      <c r="C9" s="272"/>
+      <c r="C9" s="271"/>
       <c r="D9" s="49"/>
       <c r="E9" s="49"/>
       <c r="F9" s="78">
@@ -5104,7 +5104,7 @@
     <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="227"/>
       <c r="B10" s="227"/>
-      <c r="C10" s="272"/>
+      <c r="C10" s="271"/>
       <c r="D10" s="49"/>
       <c r="E10" s="49"/>
       <c r="F10" s="78">
@@ -5154,20 +5154,20 @@
       </c>
       <c r="R10" s="49"/>
       <c r="S10" s="49"/>
-      <c r="T10" s="274" t="s">
+      <c r="T10" s="273" t="s">
         <v>28</v>
       </c>
-      <c r="U10" s="274" t="s">
+      <c r="U10" s="273" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="270" t="s">
+      <c r="V10" s="269" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" s="227"/>
       <c r="B11" s="227"/>
-      <c r="C11" s="272"/>
+      <c r="C11" s="271"/>
       <c r="D11" s="49"/>
       <c r="E11" s="49"/>
       <c r="F11" s="78">
@@ -5217,14 +5217,14 @@
       </c>
       <c r="R11" s="49"/>
       <c r="S11" s="49"/>
-      <c r="T11" s="274"/>
-      <c r="U11" s="274"/>
-      <c r="V11" s="270"/>
+      <c r="T11" s="273"/>
+      <c r="U11" s="273"/>
+      <c r="V11" s="269"/>
     </row>
     <row r="12" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="228"/>
       <c r="B12" s="228"/>
-      <c r="C12" s="273"/>
+      <c r="C12" s="272"/>
       <c r="D12" s="34"/>
       <c r="E12" s="34"/>
       <c r="F12" s="78">
@@ -5274,9 +5274,9 @@
       </c>
       <c r="R12" s="34"/>
       <c r="S12" s="34"/>
-      <c r="T12" s="274"/>
-      <c r="U12" s="274"/>
-      <c r="V12" s="270"/>
+      <c r="T12" s="273"/>
+      <c r="U12" s="273"/>
+      <c r="V12" s="269"/>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="L13" s="81">
@@ -5317,7 +5317,7 @@
         <f t="shared" si="21"/>
         <v>3</v>
       </c>
-      <c r="C17" s="271" t="str">
+      <c r="C17" s="270" t="str">
         <f t="shared" si="21"/>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -5385,7 +5385,7 @@
     <row r="18" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A18" s="35"/>
       <c r="B18" s="32"/>
-      <c r="C18" s="272"/>
+      <c r="C18" s="271"/>
       <c r="D18" s="19"/>
       <c r="E18" s="20"/>
       <c r="F18" s="78">
@@ -5439,7 +5439,7 @@
     <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" s="35"/>
       <c r="B19" s="32"/>
-      <c r="C19" s="272"/>
+      <c r="C19" s="271"/>
       <c r="D19" s="19"/>
       <c r="E19" s="20"/>
       <c r="F19" s="78">
@@ -5493,7 +5493,7 @@
     <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" s="49"/>
       <c r="B20" s="49"/>
-      <c r="C20" s="272"/>
+      <c r="C20" s="271"/>
       <c r="D20" s="49"/>
       <c r="E20" s="49"/>
       <c r="F20" s="78">
@@ -5547,7 +5547,7 @@
     <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" s="49"/>
       <c r="B21" s="49"/>
-      <c r="C21" s="272"/>
+      <c r="C21" s="271"/>
       <c r="D21" s="49"/>
       <c r="E21" s="49"/>
       <c r="F21" s="78">
@@ -5601,7 +5601,7 @@
     <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" s="49"/>
       <c r="B22" s="49"/>
-      <c r="C22" s="272"/>
+      <c r="C22" s="271"/>
       <c r="D22" s="49"/>
       <c r="E22" s="49"/>
       <c r="F22" s="78">
@@ -5655,7 +5655,7 @@
     <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" s="34"/>
       <c r="B23" s="34"/>
-      <c r="C23" s="273"/>
+      <c r="C23" s="272"/>
       <c r="D23" s="34"/>
       <c r="E23" s="34"/>
       <c r="F23" s="78">
@@ -5824,26 +5824,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="275" t="s">
+      <c r="C1" s="274" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="275"/>
+      <c r="D1" s="274"/>
       <c r="Q1" s="16"/>
     </row>
     <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="277" t="s">
+      <c r="C2" s="276" t="s">
         <v>98</v>
       </c>
-      <c r="D2" s="277"/>
-      <c r="E2" s="277"/>
-      <c r="F2" s="277"/>
-      <c r="G2" s="277"/>
-      <c r="H2" s="277"/>
-      <c r="I2" s="277"/>
-      <c r="J2" s="277"/>
-      <c r="K2" s="277"/>
-      <c r="L2" s="277"/>
-      <c r="M2" s="277"/>
+      <c r="D2" s="276"/>
+      <c r="E2" s="276"/>
+      <c r="F2" s="276"/>
+      <c r="G2" s="276"/>
+      <c r="H2" s="276"/>
+      <c r="I2" s="276"/>
+      <c r="J2" s="276"/>
+      <c r="K2" s="276"/>
+      <c r="L2" s="276"/>
+      <c r="M2" s="276"/>
       <c r="Q2" s="16"/>
     </row>
     <row r="3" spans="1:17" ht="12" customHeight="1" x14ac:dyDescent="0.3">
@@ -5905,7 +5905,7 @@
         <f>Paėmimas!B6</f>
         <v>3</v>
       </c>
-      <c r="C6" s="271" t="str">
+      <c r="C6" s="270" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -5957,7 +5957,7 @@
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="59"/>
       <c r="B7" s="23"/>
-      <c r="C7" s="272"/>
+      <c r="C7" s="271"/>
       <c r="D7" s="58">
         <f>Paėmimas!L7</f>
         <v>3.5999999999999997E-2</v>
@@ -5994,7 +5994,7 @@
     <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="59"/>
       <c r="B8" s="23"/>
-      <c r="C8" s="272"/>
+      <c r="C8" s="271"/>
       <c r="D8" s="58">
         <f>Paėmimas!L8</f>
         <v>3.5999999999999997E-2</v>
@@ -6031,7 +6031,7 @@
     <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="59"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="272"/>
+      <c r="C9" s="271"/>
       <c r="D9" s="58">
         <f>Paėmimas!L9</f>
         <v>3.5999999999999997E-2</v>
@@ -6068,7 +6068,7 @@
     <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="59"/>
       <c r="B10" s="23"/>
-      <c r="C10" s="272"/>
+      <c r="C10" s="271"/>
       <c r="D10" s="58">
         <f>Paėmimas!L10</f>
         <v>3.5999999999999997E-2</v>
@@ -6105,7 +6105,7 @@
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="59"/>
       <c r="B11" s="23"/>
-      <c r="C11" s="272"/>
+      <c r="C11" s="271"/>
       <c r="D11" s="58">
         <f>Paėmimas!L11</f>
         <v>3.3000000000000002E-2</v>
@@ -6142,7 +6142,7 @@
     <row r="12" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="61"/>
       <c r="B12" s="62"/>
-      <c r="C12" s="272"/>
+      <c r="C12" s="271"/>
       <c r="D12" s="58">
         <f>Paėmimas!L12</f>
         <v>0.03</v>
@@ -6225,7 +6225,7 @@
         <f>Paėmimas!B17</f>
         <v>3</v>
       </c>
-      <c r="C17" s="271" t="str">
+      <c r="C17" s="270" t="str">
         <f>Paėmimas!C17</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -6277,7 +6277,7 @@
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="59"/>
       <c r="B18" s="23"/>
-      <c r="C18" s="272"/>
+      <c r="C18" s="271"/>
       <c r="D18" s="58">
         <f>Paėmimas!L18</f>
         <v>3.3000000000000002E-2</v>
@@ -6314,7 +6314,7 @@
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="59"/>
       <c r="B19" s="23"/>
-      <c r="C19" s="272"/>
+      <c r="C19" s="271"/>
       <c r="D19" s="58">
         <f>Paėmimas!L19</f>
         <v>3.3000000000000002E-2</v>
@@ -6351,7 +6351,7 @@
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="59"/>
       <c r="B20" s="23"/>
-      <c r="C20" s="272"/>
+      <c r="C20" s="271"/>
       <c r="D20" s="58">
         <f>Paėmimas!L20</f>
         <v>3.5999999999999997E-2</v>
@@ -6388,7 +6388,7 @@
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="59"/>
       <c r="B21" s="23"/>
-      <c r="C21" s="272"/>
+      <c r="C21" s="271"/>
       <c r="D21" s="58">
         <f>Paėmimas!L21</f>
         <v>3.3000000000000002E-2</v>
@@ -6425,7 +6425,7 @@
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="59"/>
       <c r="B22" s="23"/>
-      <c r="C22" s="272"/>
+      <c r="C22" s="271"/>
       <c r="D22" s="58">
         <f>Paėmimas!L22</f>
         <v>3.3000000000000002E-2</v>
@@ -6462,7 +6462,7 @@
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="61"/>
       <c r="B23" s="62"/>
-      <c r="C23" s="272"/>
+      <c r="C23" s="271"/>
       <c r="D23" s="58">
         <f>Paėmimas!L23</f>
         <v>3.3000000000000002E-2</v>
@@ -6645,29 +6645,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="275" t="s">
+      <c r="C1" s="274" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="275"/>
+      <c r="D1" s="274"/>
       <c r="R1" s="16"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A2" s="277" t="s">
+      <c r="A2" s="276" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="277"/>
-      <c r="C2" s="277"/>
-      <c r="D2" s="277"/>
-      <c r="E2" s="277"/>
-      <c r="F2" s="277"/>
-      <c r="G2" s="277"/>
-      <c r="H2" s="277"/>
-      <c r="I2" s="277"/>
-      <c r="J2" s="277"/>
-      <c r="K2" s="277"/>
-      <c r="L2" s="277"/>
-      <c r="M2" s="277"/>
-      <c r="N2" s="277"/>
+      <c r="B2" s="276"/>
+      <c r="C2" s="276"/>
+      <c r="D2" s="276"/>
+      <c r="E2" s="276"/>
+      <c r="F2" s="276"/>
+      <c r="G2" s="276"/>
+      <c r="H2" s="276"/>
+      <c r="I2" s="276"/>
+      <c r="J2" s="276"/>
+      <c r="K2" s="276"/>
+      <c r="L2" s="276"/>
+      <c r="M2" s="276"/>
+      <c r="N2" s="276"/>
       <c r="O2" s="156"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
@@ -6738,7 +6738,7 @@
         <f>Svėrimas!A6</f>
         <v>3</v>
       </c>
-      <c r="C6" s="278" t="str">
+      <c r="C6" s="277" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -6797,7 +6797,7 @@
     <row r="7" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="66"/>
       <c r="B7" s="67"/>
-      <c r="C7" s="278"/>
+      <c r="C7" s="277"/>
       <c r="D7" s="68"/>
       <c r="E7" s="127"/>
       <c r="F7" s="129"/>
@@ -6815,7 +6815,7 @@
     <row r="8" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="76"/>
       <c r="B8" s="65"/>
-      <c r="C8" s="279"/>
+      <c r="C8" s="278"/>
       <c r="D8" s="68"/>
       <c r="E8" s="127"/>
       <c r="F8" s="129"/>
@@ -6871,76 +6871,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="275" t="s">
+      <c r="C1" s="274" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="275"/>
-      <c r="E1" s="275"/>
-      <c r="F1" s="275"/>
+      <c r="D1" s="274"/>
+      <c r="E1" s="274"/>
+      <c r="F1" s="274"/>
     </row>
     <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="277" t="s">
+      <c r="A2" s="276" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="277"/>
-      <c r="C2" s="277"/>
-      <c r="D2" s="277"/>
-      <c r="E2" s="277"/>
-      <c r="F2" s="277"/>
-      <c r="G2" s="277"/>
-      <c r="H2" s="277"/>
-      <c r="I2" s="277"/>
-      <c r="J2" s="277"/>
-      <c r="K2" s="277"/>
-      <c r="L2" s="277"/>
-      <c r="M2" s="277"/>
-      <c r="N2" s="277"/>
-      <c r="O2" s="277"/>
+      <c r="B2" s="276"/>
+      <c r="C2" s="276"/>
+      <c r="D2" s="276"/>
+      <c r="E2" s="276"/>
+      <c r="F2" s="276"/>
+      <c r="G2" s="276"/>
+      <c r="H2" s="276"/>
+      <c r="I2" s="276"/>
+      <c r="J2" s="276"/>
+      <c r="K2" s="276"/>
+      <c r="L2" s="276"/>
+      <c r="M2" s="276"/>
+      <c r="N2" s="276"/>
+      <c r="O2" s="276"/>
     </row>
     <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="281" t="s">
+      <c r="A4" s="280" t="s">
         <v>80</v>
       </c>
-      <c r="B4" s="281" t="s">
+      <c r="B4" s="280" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="292" t="s">
+      <c r="C4" s="291" t="s">
         <v>81</v>
       </c>
-      <c r="D4" s="292" t="s">
+      <c r="D4" s="291" t="s">
         <v>82</v>
       </c>
-      <c r="E4" s="292" t="s">
+      <c r="E4" s="291" t="s">
         <v>83</v>
       </c>
-      <c r="F4" s="292"/>
-      <c r="G4" s="292"/>
-      <c r="H4" s="292" t="s">
+      <c r="F4" s="291"/>
+      <c r="G4" s="291"/>
+      <c r="H4" s="291" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="285" t="s">
+      <c r="I4" s="284" t="s">
         <v>84</v>
       </c>
-      <c r="J4" s="280" t="s">
+      <c r="J4" s="279" t="s">
         <v>85</v>
       </c>
-      <c r="K4" s="280"/>
-      <c r="L4" s="280"/>
-      <c r="M4" s="287" t="s">
+      <c r="K4" s="279"/>
+      <c r="L4" s="279"/>
+      <c r="M4" s="286" t="s">
         <v>86</v>
       </c>
-      <c r="N4" s="280" t="s">
+      <c r="N4" s="279" t="s">
         <v>13</v>
       </c>
-      <c r="O4" s="283" t="s">
+      <c r="O4" s="282" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="282"/>
-      <c r="B5" s="282"/>
-      <c r="C5" s="293"/>
-      <c r="D5" s="292"/>
+      <c r="A5" s="281"/>
+      <c r="B5" s="281"/>
+      <c r="C5" s="292"/>
+      <c r="D5" s="291"/>
       <c r="E5" s="146">
         <v>1</v>
       </c>
@@ -6950,8 +6950,8 @@
       <c r="G5" s="146">
         <v>3</v>
       </c>
-      <c r="H5" s="292"/>
-      <c r="I5" s="286"/>
+      <c r="H5" s="291"/>
+      <c r="I5" s="285"/>
       <c r="J5" s="12">
         <v>1</v>
       </c>
@@ -6961,16 +6961,16 @@
       <c r="L5" s="12">
         <v>3</v>
       </c>
-      <c r="M5" s="288"/>
-      <c r="N5" s="280"/>
-      <c r="O5" s="284"/>
+      <c r="M5" s="287"/>
+      <c r="N5" s="279"/>
+      <c r="O5" s="283"/>
     </row>
     <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="170" t="str">
         <f>Paėmimas!B6</f>
         <v>3</v>
       </c>
-      <c r="B6" s="289" t="str">
+      <c r="B6" s="288" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -7019,7 +7019,7 @@
     </row>
     <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="32"/>
-      <c r="B7" s="290"/>
+      <c r="B7" s="289"/>
       <c r="C7" s="31"/>
       <c r="D7" s="28"/>
       <c r="E7" s="231"/>
@@ -7039,7 +7039,7 @@
     </row>
     <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="32"/>
-      <c r="B8" s="290"/>
+      <c r="B8" s="289"/>
       <c r="C8" s="31"/>
       <c r="D8" s="106"/>
       <c r="E8" s="231"/>
@@ -7059,7 +7059,7 @@
     </row>
     <row r="9" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A9" s="32"/>
-      <c r="B9" s="290"/>
+      <c r="B9" s="289"/>
       <c r="C9" s="31">
         <v>2</v>
       </c>
@@ -7096,7 +7096,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="32"/>
-      <c r="B10" s="290"/>
+      <c r="B10" s="289"/>
       <c r="C10" s="31"/>
       <c r="D10" s="106"/>
       <c r="E10" s="231"/>
@@ -7113,7 +7113,7 @@
     </row>
     <row r="11" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A11" s="32"/>
-      <c r="B11" s="290"/>
+      <c r="B11" s="289"/>
       <c r="C11" s="31">
         <v>41</v>
       </c>
@@ -7149,7 +7149,7 @@
     </row>
     <row r="12" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="32"/>
-      <c r="B12" s="290"/>
+      <c r="B12" s="289"/>
       <c r="C12" s="138" t="s">
         <v>41</v>
       </c>
@@ -7185,7 +7185,7 @@
     </row>
     <row r="13" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A13" s="32"/>
-      <c r="B13" s="290"/>
+      <c r="B13" s="289"/>
       <c r="C13" s="139" t="s">
         <v>42</v>
       </c>
@@ -7221,7 +7221,7 @@
     </row>
     <row r="14" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A14" s="32"/>
-      <c r="B14" s="290"/>
+      <c r="B14" s="289"/>
       <c r="C14" s="139" t="s">
         <v>43</v>
       </c>
@@ -7257,7 +7257,7 @@
     </row>
     <row r="15" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A15" s="32"/>
-      <c r="B15" s="290"/>
+      <c r="B15" s="289"/>
       <c r="C15" s="140" t="s">
         <v>44</v>
       </c>
@@ -7293,7 +7293,7 @@
     </row>
     <row r="16" spans="1:16" ht="32.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="22"/>
-      <c r="B16" s="291"/>
+      <c r="B16" s="290"/>
       <c r="C16" s="31"/>
       <c r="D16" s="109"/>
       <c r="E16" s="21"/>
@@ -7367,12 +7367,12 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="243" t="s">
+      <c r="A3" s="293" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="243"/>
-      <c r="C3" s="243"/>
-      <c r="D3" s="243"/>
+      <c r="B3" s="293"/>
+      <c r="C3" s="293"/>
+      <c r="D3" s="293"/>
     </row>
     <row r="5" spans="1:4" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="131" t="s">

</xml_diff>

<commit_message>
Paleista Pradiniai3Funkcija.py, perkelia O2, CO2, temperatura
</commit_message>
<xml_diff>
--- a/Ivestis1.xlsx
+++ b/Ivestis1.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="130" documentId="13_ncr:1_{01443EB8-4D64-407F-8533-569B30C1461B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57E278BD-8C50-4613-80CC-64D50D242CD1}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="1" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="3" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Compatibility Report" sheetId="4" state="hidden" r:id="rId1"/>
@@ -2630,6 +2630,98 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="30" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -2662,98 +2754,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="30" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3258,31 +3258,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="D3" s="258" t="s">
+      <c r="D3" s="249" t="s">
         <v>105</v>
       </c>
-      <c r="E3" s="258"/>
-      <c r="F3" s="258"/>
-      <c r="G3" s="258"/>
-      <c r="H3" s="258"/>
-      <c r="I3" s="258"/>
-      <c r="J3" s="258"/>
-      <c r="K3" s="258"/>
-      <c r="L3" s="258"/>
-      <c r="M3" s="258"/>
-      <c r="N3" s="258"/>
-      <c r="O3" s="258"/>
-      <c r="P3" s="258"/>
-      <c r="Q3" s="258"/>
-      <c r="R3" s="258"/>
-      <c r="S3" s="258"/>
-      <c r="T3" s="258"/>
-      <c r="U3" s="258"/>
-      <c r="V3" s="258"/>
-      <c r="W3" s="258"/>
-      <c r="X3" s="258"/>
-      <c r="Y3" s="258"/>
-      <c r="Z3" s="258"/>
+      <c r="E3" s="249"/>
+      <c r="F3" s="249"/>
+      <c r="G3" s="249"/>
+      <c r="H3" s="249"/>
+      <c r="I3" s="249"/>
+      <c r="J3" s="249"/>
+      <c r="K3" s="249"/>
+      <c r="L3" s="249"/>
+      <c r="M3" s="249"/>
+      <c r="N3" s="249"/>
+      <c r="O3" s="249"/>
+      <c r="P3" s="249"/>
+      <c r="Q3" s="249"/>
+      <c r="R3" s="249"/>
+      <c r="S3" s="249"/>
+      <c r="T3" s="249"/>
+      <c r="U3" s="249"/>
+      <c r="V3" s="249"/>
+      <c r="W3" s="249"/>
+      <c r="X3" s="249"/>
+      <c r="Y3" s="249"/>
+      <c r="Z3" s="249"/>
     </row>
     <row r="5" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
@@ -3371,13 +3371,13 @@
       </c>
     </row>
     <row r="6" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="259">
+      <c r="A6" s="250">
         <v>46210</v>
       </c>
-      <c r="B6" s="262">
+      <c r="B6" s="253">
         <v>7</v>
       </c>
-      <c r="C6" s="263" t="s">
+      <c r="C6" s="254" t="s">
         <v>134</v>
       </c>
       <c r="D6" s="143">
@@ -3463,14 +3463,14 @@
         <f>Aerodinamika!G23</f>
         <v>1.2973599999999998</v>
       </c>
-      <c r="AB6" s="256" t="s">
+      <c r="AB6" s="247" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="260"/>
-      <c r="B7" s="260"/>
-      <c r="C7" s="264"/>
+      <c r="A7" s="251"/>
+      <c r="B7" s="251"/>
+      <c r="C7" s="255"/>
       <c r="D7" s="143">
         <v>2</v>
       </c>
@@ -3550,12 +3550,12 @@
         <f>O6*X7</f>
         <v>0.34775490281286214</v>
       </c>
-      <c r="AB7" s="257"/>
+      <c r="AB7" s="248"/>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="260"/>
-      <c r="B8" s="260"/>
-      <c r="C8" s="264"/>
+      <c r="A8" s="251"/>
+      <c r="B8" s="251"/>
+      <c r="C8" s="255"/>
       <c r="D8" s="166">
         <v>3</v>
       </c>
@@ -3601,9 +3601,9 @@
       <c r="S8" s="142"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A9" s="260"/>
-      <c r="B9" s="260"/>
-      <c r="C9" s="264"/>
+      <c r="A9" s="251"/>
+      <c r="B9" s="251"/>
+      <c r="C9" s="255"/>
       <c r="D9" s="143">
         <v>4</v>
       </c>
@@ -3653,9 +3653,9 @@
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A10" s="260"/>
-      <c r="B10" s="260"/>
-      <c r="C10" s="264"/>
+      <c r="A10" s="251"/>
+      <c r="B10" s="251"/>
+      <c r="C10" s="255"/>
       <c r="D10" s="143">
         <v>5</v>
       </c>
@@ -3694,9 +3694,9 @@
       <c r="N10" s="209"/>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A11" s="260"/>
-      <c r="B11" s="260"/>
-      <c r="C11" s="264"/>
+      <c r="A11" s="251"/>
+      <c r="B11" s="251"/>
+      <c r="C11" s="255"/>
       <c r="D11" s="166">
         <v>6</v>
       </c>
@@ -3735,9 +3735,9 @@
       <c r="N11" s="209"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A12" s="260"/>
-      <c r="B12" s="260"/>
-      <c r="C12" s="264"/>
+      <c r="A12" s="251"/>
+      <c r="B12" s="251"/>
+      <c r="C12" s="255"/>
       <c r="D12" s="143">
         <v>7</v>
       </c>
@@ -3776,9 +3776,9 @@
       <c r="N12" s="209"/>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A13" s="260"/>
-      <c r="B13" s="260"/>
-      <c r="C13" s="264"/>
+      <c r="A13" s="251"/>
+      <c r="B13" s="251"/>
+      <c r="C13" s="255"/>
       <c r="D13" s="143">
         <v>8</v>
       </c>
@@ -3818,9 +3818,9 @@
       <c r="O13" s="137"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A14" s="260"/>
-      <c r="B14" s="260"/>
-      <c r="C14" s="264"/>
+      <c r="A14" s="251"/>
+      <c r="B14" s="251"/>
+      <c r="C14" s="255"/>
       <c r="D14" s="166">
         <v>9</v>
       </c>
@@ -3863,9 +3863,9 @@
       <c r="U14" s="38"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A15" s="260"/>
-      <c r="B15" s="260"/>
-      <c r="C15" s="264"/>
+      <c r="A15" s="251"/>
+      <c r="B15" s="251"/>
+      <c r="C15" s="255"/>
       <c r="D15" s="143">
         <v>10</v>
       </c>
@@ -3908,9 +3908,9 @@
       <c r="U15" s="38"/>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A16" s="260"/>
-      <c r="B16" s="260"/>
-      <c r="C16" s="264"/>
+      <c r="A16" s="251"/>
+      <c r="B16" s="251"/>
+      <c r="C16" s="255"/>
       <c r="D16" s="143">
         <v>11</v>
       </c>
@@ -3953,9 +3953,9 @@
       <c r="U16" s="38"/>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A17" s="260"/>
-      <c r="B17" s="260"/>
-      <c r="C17" s="264"/>
+      <c r="A17" s="251"/>
+      <c r="B17" s="251"/>
+      <c r="C17" s="255"/>
       <c r="D17" s="166">
         <v>12</v>
       </c>
@@ -3998,9 +3998,9 @@
       <c r="U17" s="38"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A18" s="260"/>
-      <c r="B18" s="260"/>
-      <c r="C18" s="264"/>
+      <c r="A18" s="251"/>
+      <c r="B18" s="251"/>
+      <c r="C18" s="255"/>
       <c r="D18" s="143">
         <v>13</v>
       </c>
@@ -4043,9 +4043,9 @@
       <c r="U18" s="38"/>
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A19" s="260"/>
-      <c r="B19" s="260"/>
-      <c r="C19" s="264"/>
+      <c r="A19" s="251"/>
+      <c r="B19" s="251"/>
+      <c r="C19" s="255"/>
       <c r="D19" s="143">
         <v>14</v>
       </c>
@@ -4088,9 +4088,9 @@
       <c r="U19" s="38"/>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A20" s="260"/>
-      <c r="B20" s="260"/>
-      <c r="C20" s="264"/>
+      <c r="A20" s="251"/>
+      <c r="B20" s="251"/>
+      <c r="C20" s="255"/>
       <c r="D20" s="166">
         <v>15</v>
       </c>
@@ -4133,9 +4133,9 @@
       <c r="U20" s="38"/>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A21" s="260"/>
-      <c r="B21" s="260"/>
-      <c r="C21" s="264"/>
+      <c r="A21" s="251"/>
+      <c r="B21" s="251"/>
+      <c r="C21" s="255"/>
       <c r="D21" s="143">
         <v>16</v>
       </c>
@@ -4178,9 +4178,9 @@
       <c r="U21" s="38"/>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A22" s="261"/>
-      <c r="B22" s="261"/>
-      <c r="C22" s="265"/>
+      <c r="A22" s="252"/>
+      <c r="B22" s="252"/>
+      <c r="C22" s="256"/>
       <c r="D22" s="143">
         <v>17</v>
       </c>
@@ -4284,11 +4284,11 @@
         <v>0</v>
       </c>
       <c r="N24" s="71"/>
-      <c r="O24" s="266" t="s">
+      <c r="O24" s="257" t="s">
         <v>131</v>
       </c>
-      <c r="P24" s="267"/>
-      <c r="Q24" s="267"/>
+      <c r="P24" s="258"/>
+      <c r="Q24" s="258"/>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="177"/>
@@ -4323,30 +4323,30 @@
       <c r="A28" s="177"/>
       <c r="B28" s="177"/>
       <c r="C28" s="177"/>
-      <c r="D28" s="268" t="s">
+      <c r="D28" s="259" t="s">
         <v>133</v>
       </c>
-      <c r="E28" s="258"/>
-      <c r="F28" s="258"/>
-      <c r="G28" s="258"/>
-      <c r="H28" s="258"/>
-      <c r="I28" s="258"/>
-      <c r="J28" s="258"/>
-      <c r="K28" s="258"/>
-      <c r="L28" s="258"/>
-      <c r="M28" s="258"/>
-      <c r="N28" s="258"/>
-      <c r="O28" s="258"/>
-      <c r="P28" s="258"/>
-      <c r="Q28" s="258"/>
-      <c r="R28" s="258"/>
-      <c r="S28" s="258"/>
-      <c r="T28" s="258"/>
-      <c r="U28" s="258"/>
-      <c r="V28" s="258"/>
-      <c r="W28" s="258"/>
-      <c r="X28" s="258"/>
-      <c r="Y28" s="258"/>
+      <c r="E28" s="249"/>
+      <c r="F28" s="249"/>
+      <c r="G28" s="249"/>
+      <c r="H28" s="249"/>
+      <c r="I28" s="249"/>
+      <c r="J28" s="249"/>
+      <c r="K28" s="249"/>
+      <c r="L28" s="249"/>
+      <c r="M28" s="249"/>
+      <c r="N28" s="249"/>
+      <c r="O28" s="249"/>
+      <c r="P28" s="249"/>
+      <c r="Q28" s="249"/>
+      <c r="R28" s="249"/>
+      <c r="S28" s="249"/>
+      <c r="T28" s="249"/>
+      <c r="U28" s="249"/>
+      <c r="V28" s="249"/>
+      <c r="W28" s="249"/>
+      <c r="X28" s="249"/>
+      <c r="Y28" s="249"/>
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="177"/>
@@ -4451,9 +4451,9 @@
       </c>
     </row>
     <row r="31" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="269"/>
-      <c r="B31" s="269"/>
-      <c r="C31" s="269"/>
+      <c r="A31" s="260"/>
+      <c r="B31" s="260"/>
+      <c r="C31" s="260"/>
       <c r="D31" s="143">
         <v>5</v>
       </c>
@@ -4528,12 +4528,12 @@
       <c r="AA31" s="187">
         <v>1.29</v>
       </c>
-      <c r="AB31" s="256"/>
+      <c r="AB31" s="247"/>
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A32" s="270"/>
-      <c r="B32" s="270"/>
-      <c r="C32" s="270"/>
+      <c r="A32" s="261"/>
+      <c r="B32" s="261"/>
+      <c r="C32" s="261"/>
       <c r="D32" s="143">
         <v>14</v>
       </c>
@@ -4602,12 +4602,12 @@
         <f>O31*X32</f>
         <v>0.90295018924227777</v>
       </c>
-      <c r="AB32" s="257"/>
+      <c r="AB32" s="248"/>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A33" s="270"/>
-      <c r="B33" s="270"/>
-      <c r="C33" s="270"/>
+      <c r="A33" s="261"/>
+      <c r="B33" s="261"/>
+      <c r="C33" s="261"/>
       <c r="D33" s="166">
         <v>24</v>
       </c>
@@ -4644,9 +4644,9 @@
       <c r="S33" s="142"/>
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A34" s="270"/>
-      <c r="B34" s="270"/>
-      <c r="C34" s="270"/>
+      <c r="A34" s="261"/>
+      <c r="B34" s="261"/>
+      <c r="C34" s="261"/>
       <c r="D34" s="143">
         <v>33</v>
       </c>
@@ -4687,9 +4687,9 @@
       </c>
     </row>
     <row r="35" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A35" s="270"/>
-      <c r="B35" s="270"/>
-      <c r="C35" s="270"/>
+      <c r="A35" s="261"/>
+      <c r="B35" s="261"/>
+      <c r="C35" s="261"/>
       <c r="D35" s="143">
         <v>42</v>
       </c>
@@ -4719,9 +4719,9 @@
       <c r="N35" s="149"/>
     </row>
     <row r="36" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A36" s="270"/>
-      <c r="B36" s="270"/>
-      <c r="C36" s="270"/>
+      <c r="A36" s="261"/>
+      <c r="B36" s="261"/>
+      <c r="C36" s="261"/>
       <c r="D36" s="143">
         <v>52</v>
       </c>
@@ -4751,9 +4751,9 @@
       <c r="N36" s="149"/>
     </row>
     <row r="37" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A37" s="270"/>
-      <c r="B37" s="270"/>
-      <c r="C37" s="270"/>
+      <c r="A37" s="261"/>
+      <c r="B37" s="261"/>
+      <c r="C37" s="261"/>
       <c r="D37" s="143">
         <v>61</v>
       </c>
@@ -4783,9 +4783,9 @@
       <c r="N37" s="149"/>
     </row>
     <row r="38" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A38" s="270"/>
-      <c r="B38" s="270"/>
-      <c r="C38" s="270"/>
+      <c r="A38" s="261"/>
+      <c r="B38" s="261"/>
+      <c r="C38" s="261"/>
       <c r="D38" s="143">
         <v>71</v>
       </c>
@@ -4816,9 +4816,9 @@
       <c r="O38" s="137"/>
     </row>
     <row r="39" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A39" s="270"/>
-      <c r="B39" s="270"/>
-      <c r="C39" s="270"/>
+      <c r="A39" s="261"/>
+      <c r="B39" s="261"/>
+      <c r="C39" s="261"/>
       <c r="D39" s="143">
         <v>80</v>
       </c>
@@ -4852,9 +4852,9 @@
       <c r="U39" s="38"/>
     </row>
     <row r="40" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A40" s="270"/>
-      <c r="B40" s="270"/>
-      <c r="C40" s="270"/>
+      <c r="A40" s="261"/>
+      <c r="B40" s="261"/>
+      <c r="C40" s="261"/>
       <c r="D40" s="143">
         <v>89</v>
       </c>
@@ -4884,9 +4884,9 @@
       <c r="N40" s="143"/>
     </row>
     <row r="41" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A41" s="270"/>
-      <c r="B41" s="270"/>
-      <c r="C41" s="270"/>
+      <c r="A41" s="261"/>
+      <c r="B41" s="261"/>
+      <c r="C41" s="261"/>
       <c r="D41" s="143">
         <v>99</v>
       </c>
@@ -4916,9 +4916,9 @@
       <c r="N41" s="143"/>
     </row>
     <row r="42" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A42" s="270"/>
-      <c r="B42" s="270"/>
-      <c r="C42" s="270"/>
+      <c r="A42" s="261"/>
+      <c r="B42" s="261"/>
+      <c r="C42" s="261"/>
       <c r="D42" s="143">
         <v>108</v>
       </c>
@@ -4948,9 +4948,9 @@
       <c r="N42" s="143"/>
     </row>
     <row r="43" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A43" s="270"/>
-      <c r="B43" s="270"/>
-      <c r="C43" s="270"/>
+      <c r="A43" s="261"/>
+      <c r="B43" s="261"/>
+      <c r="C43" s="261"/>
       <c r="D43" s="143">
         <v>118</v>
       </c>
@@ -4980,9 +4980,9 @@
       <c r="N43" s="143"/>
     </row>
     <row r="44" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A44" s="270"/>
-      <c r="B44" s="270"/>
-      <c r="C44" s="270"/>
+      <c r="A44" s="261"/>
+      <c r="B44" s="261"/>
+      <c r="C44" s="261"/>
       <c r="D44" s="143">
         <v>127</v>
       </c>
@@ -5012,9 +5012,9 @@
       <c r="N44" s="143"/>
     </row>
     <row r="45" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A45" s="270"/>
-      <c r="B45" s="270"/>
-      <c r="C45" s="270"/>
+      <c r="A45" s="261"/>
+      <c r="B45" s="261"/>
+      <c r="C45" s="261"/>
       <c r="D45" s="143">
         <v>136</v>
       </c>
@@ -5044,9 +5044,9 @@
       <c r="N45" s="143"/>
     </row>
     <row r="46" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A46" s="270"/>
-      <c r="B46" s="270"/>
-      <c r="C46" s="270"/>
+      <c r="A46" s="261"/>
+      <c r="B46" s="261"/>
+      <c r="C46" s="261"/>
       <c r="D46" s="143">
         <v>146</v>
       </c>
@@ -5076,9 +5076,9 @@
       <c r="N46" s="143"/>
     </row>
     <row r="47" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A47" s="271"/>
-      <c r="B47" s="271"/>
-      <c r="C47" s="271"/>
+      <c r="A47" s="262"/>
+      <c r="B47" s="262"/>
+      <c r="C47" s="262"/>
       <c r="D47" s="143">
         <v>155</v>
       </c>
@@ -5167,18 +5167,18 @@
       <c r="I2" s="10"/>
     </row>
     <row r="3" spans="1:12" ht="15" x14ac:dyDescent="0.3">
-      <c r="A3" s="272" t="s">
+      <c r="A3" s="263" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="272"/>
-      <c r="C3" s="272"/>
-      <c r="D3" s="272"/>
-      <c r="E3" s="272"/>
-      <c r="F3" s="272"/>
-      <c r="G3" s="272"/>
-      <c r="H3" s="272"/>
-      <c r="I3" s="272"/>
-      <c r="J3" s="272"/>
+      <c r="B3" s="263"/>
+      <c r="C3" s="263"/>
+      <c r="D3" s="263"/>
+      <c r="E3" s="263"/>
+      <c r="F3" s="263"/>
+      <c r="G3" s="263"/>
+      <c r="H3" s="263"/>
+      <c r="I3" s="263"/>
+      <c r="J3" s="263"/>
     </row>
     <row r="4" spans="1:12" ht="14" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
@@ -5325,46 +5325,46 @@
       <c r="L10" s="45"/>
     </row>
     <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H11" s="273" t="s">
+      <c r="H11" s="264" t="s">
         <v>29</v>
       </c>
-      <c r="I11" s="276" t="s">
+      <c r="I11" s="267" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H12" s="274"/>
-      <c r="I12" s="277"/>
+      <c r="H12" s="265"/>
+      <c r="I12" s="268"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H13" s="274"/>
-      <c r="I13" s="277"/>
+      <c r="H13" s="265"/>
+      <c r="I13" s="268"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H14" s="274"/>
-      <c r="I14" s="277"/>
+      <c r="H14" s="265"/>
+      <c r="I14" s="268"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H15" s="274"/>
-      <c r="I15" s="277"/>
+      <c r="H15" s="265"/>
+      <c r="I15" s="268"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H16" s="274"/>
-      <c r="I16" s="277"/>
+      <c r="H16" s="265"/>
+      <c r="I16" s="268"/>
     </row>
     <row r="17" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H17" s="274"/>
-      <c r="I17" s="277"/>
+      <c r="H17" s="265"/>
+      <c r="I17" s="268"/>
     </row>
     <row r="18" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H18" s="275"/>
-      <c r="I18" s="277"/>
+      <c r="H18" s="266"/>
+      <c r="I18" s="268"/>
     </row>
     <row r="19" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="I19" s="277"/>
+      <c r="I19" s="268"/>
     </row>
     <row r="20" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="I20" s="278"/>
+      <c r="I20" s="269"/>
     </row>
     <row r="23" spans="8:9" ht="14" x14ac:dyDescent="0.3">
       <c r="I23" s="52"/>
@@ -5425,35 +5425,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="251" t="s">
+      <c r="C1" s="274" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="251"/>
+      <c r="D1" s="274"/>
       <c r="E1" s="15"/>
       <c r="S1" s="80"/>
     </row>
     <row r="2" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="252" t="s">
+      <c r="A2" s="275" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="252"/>
-      <c r="C2" s="252"/>
-      <c r="D2" s="252"/>
-      <c r="E2" s="252"/>
-      <c r="F2" s="252"/>
-      <c r="G2" s="252"/>
-      <c r="H2" s="252"/>
-      <c r="I2" s="252"/>
-      <c r="J2" s="252"/>
-      <c r="K2" s="252"/>
-      <c r="L2" s="252"/>
-      <c r="M2" s="252"/>
-      <c r="N2" s="252"/>
-      <c r="O2" s="252"/>
-      <c r="P2" s="252"/>
-      <c r="Q2" s="252"/>
-      <c r="R2" s="252"/>
-      <c r="S2" s="252"/>
+      <c r="B2" s="275"/>
+      <c r="C2" s="275"/>
+      <c r="D2" s="275"/>
+      <c r="E2" s="275"/>
+      <c r="F2" s="275"/>
+      <c r="G2" s="275"/>
+      <c r="H2" s="275"/>
+      <c r="I2" s="275"/>
+      <c r="J2" s="275"/>
+      <c r="K2" s="275"/>
+      <c r="L2" s="275"/>
+      <c r="M2" s="275"/>
+      <c r="N2" s="275"/>
+      <c r="O2" s="275"/>
+      <c r="P2" s="275"/>
+      <c r="Q2" s="275"/>
+      <c r="R2" s="275"/>
+      <c r="S2" s="275"/>
     </row>
     <row r="3" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="81"/>
@@ -5562,7 +5562,7 @@
       <c r="B6" s="49">
         <v>1</v>
       </c>
-      <c r="C6" s="253" t="str">
+      <c r="C6" s="276" t="str">
         <f>Greitis!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -5642,7 +5642,7 @@
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="36"/>
       <c r="B7" s="33"/>
-      <c r="C7" s="254"/>
+      <c r="C7" s="277"/>
       <c r="D7" s="17"/>
       <c r="E7" s="18"/>
       <c r="F7" s="211">
@@ -5713,7 +5713,7 @@
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" s="36"/>
       <c r="B8" s="33"/>
-      <c r="C8" s="254"/>
+      <c r="C8" s="277"/>
       <c r="D8" s="17"/>
       <c r="E8" s="18"/>
       <c r="F8" s="211">
@@ -5784,7 +5784,7 @@
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="36"/>
       <c r="B9" s="33"/>
-      <c r="C9" s="254"/>
+      <c r="C9" s="277"/>
       <c r="D9" s="85"/>
       <c r="E9" s="85"/>
       <c r="F9" s="211">
@@ -5858,7 +5858,7 @@
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="85"/>
       <c r="B10" s="85"/>
-      <c r="C10" s="254"/>
+      <c r="C10" s="277"/>
       <c r="D10" s="85"/>
       <c r="E10" s="85"/>
       <c r="F10" s="211">
@@ -5908,13 +5908,13 @@
       </c>
       <c r="R10" s="85"/>
       <c r="S10" s="85"/>
-      <c r="T10" s="248" t="s">
+      <c r="T10" s="271" t="s">
         <v>31</v>
       </c>
-      <c r="U10" s="248" t="s">
+      <c r="U10" s="271" t="s">
         <v>32</v>
       </c>
-      <c r="V10" s="247" t="s">
+      <c r="V10" s="270" t="s">
         <v>36</v>
       </c>
       <c r="X10" s="205">
@@ -5929,7 +5929,7 @@
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="85"/>
       <c r="B11" s="85"/>
-      <c r="C11" s="254"/>
+      <c r="C11" s="277"/>
       <c r="D11" s="85"/>
       <c r="E11" s="85"/>
       <c r="F11" s="211">
@@ -5979,9 +5979,9 @@
       </c>
       <c r="R11" s="85"/>
       <c r="S11" s="85"/>
-      <c r="T11" s="249"/>
-      <c r="U11" s="249"/>
-      <c r="V11" s="247"/>
+      <c r="T11" s="272"/>
+      <c r="U11" s="272"/>
+      <c r="V11" s="270"/>
       <c r="X11" s="205">
         <f>Greitis!E11</f>
         <v>0.14000000000000001</v>
@@ -5994,7 +5994,7 @@
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="85"/>
       <c r="B12" s="85"/>
-      <c r="C12" s="254"/>
+      <c r="C12" s="277"/>
       <c r="D12" s="85"/>
       <c r="E12" s="85"/>
       <c r="F12" s="211">
@@ -6044,9 +6044,9 @@
       </c>
       <c r="R12" s="85"/>
       <c r="S12" s="85"/>
-      <c r="T12" s="250"/>
-      <c r="U12" s="250"/>
-      <c r="V12" s="247"/>
+      <c r="T12" s="273"/>
+      <c r="U12" s="273"/>
+      <c r="V12" s="270"/>
       <c r="X12" s="205">
         <f>Greitis!E12</f>
         <v>0.14000000000000001</v>
@@ -6059,7 +6059,7 @@
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="85"/>
       <c r="B13" s="85"/>
-      <c r="C13" s="254"/>
+      <c r="C13" s="277"/>
       <c r="D13" s="85"/>
       <c r="E13" s="85"/>
       <c r="F13" s="211">
@@ -6121,7 +6121,7 @@
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="85"/>
       <c r="B14" s="85"/>
-      <c r="C14" s="254"/>
+      <c r="C14" s="277"/>
       <c r="D14" s="85"/>
       <c r="E14" s="85"/>
       <c r="F14" s="211">
@@ -6183,7 +6183,7 @@
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="85"/>
       <c r="B15" s="85"/>
-      <c r="C15" s="254"/>
+      <c r="C15" s="277"/>
       <c r="D15" s="85"/>
       <c r="E15" s="85"/>
       <c r="F15" s="211">
@@ -6245,7 +6245,7 @@
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="85"/>
       <c r="B16" s="85"/>
-      <c r="C16" s="254"/>
+      <c r="C16" s="277"/>
       <c r="D16" s="85"/>
       <c r="E16" s="85"/>
       <c r="F16" s="211">
@@ -6307,7 +6307,7 @@
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" s="85"/>
       <c r="B17" s="85"/>
-      <c r="C17" s="254"/>
+      <c r="C17" s="277"/>
       <c r="D17" s="85"/>
       <c r="E17" s="85"/>
       <c r="F17" s="211">
@@ -6369,7 +6369,7 @@
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" s="85"/>
       <c r="B18" s="85"/>
-      <c r="C18" s="254"/>
+      <c r="C18" s="277"/>
       <c r="D18" s="85"/>
       <c r="E18" s="85"/>
       <c r="F18" s="211">
@@ -6431,7 +6431,7 @@
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" s="85"/>
       <c r="B19" s="85"/>
-      <c r="C19" s="254"/>
+      <c r="C19" s="277"/>
       <c r="D19" s="85"/>
       <c r="E19" s="85"/>
       <c r="F19" s="211">
@@ -6493,7 +6493,7 @@
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" s="85"/>
       <c r="B20" s="85"/>
-      <c r="C20" s="254"/>
+      <c r="C20" s="277"/>
       <c r="D20" s="85"/>
       <c r="E20" s="85"/>
       <c r="F20" s="211">
@@ -6555,7 +6555,7 @@
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" s="85"/>
       <c r="B21" s="85"/>
-      <c r="C21" s="254"/>
+      <c r="C21" s="277"/>
       <c r="D21" s="85"/>
       <c r="E21" s="85"/>
       <c r="F21" s="211">
@@ -6617,7 +6617,7 @@
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" s="86"/>
       <c r="B22" s="86"/>
-      <c r="C22" s="255"/>
+      <c r="C22" s="278"/>
       <c r="D22" s="86"/>
       <c r="E22" s="86"/>
       <c r="F22" s="211">
@@ -6763,10 +6763,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="251" t="s">
+      <c r="C1" s="274" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="251"/>
+      <c r="D1" s="274"/>
       <c r="Q1" s="16"/>
     </row>
     <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -6844,7 +6844,7 @@
         <f>Paėmimas!B6</f>
         <v>1</v>
       </c>
-      <c r="C6" s="253" t="str">
+      <c r="C6" s="276" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -6896,7 +6896,7 @@
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="54"/>
       <c r="B7" s="21"/>
-      <c r="C7" s="254"/>
+      <c r="C7" s="277"/>
       <c r="D7" s="217">
         <f>Paėmimas!L7</f>
         <v>0.03</v>
@@ -6933,7 +6933,7 @@
     <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="54"/>
       <c r="B8" s="21"/>
-      <c r="C8" s="254"/>
+      <c r="C8" s="277"/>
       <c r="D8" s="217">
         <f>Paėmimas!L8</f>
         <v>0.03</v>
@@ -6970,7 +6970,7 @@
     <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="54"/>
       <c r="B9" s="21"/>
-      <c r="C9" s="254"/>
+      <c r="C9" s="277"/>
       <c r="D9" s="217">
         <f>Paėmimas!L9</f>
         <v>0.03</v>
@@ -7007,7 +7007,7 @@
     <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="54"/>
       <c r="B10" s="21"/>
-      <c r="C10" s="254"/>
+      <c r="C10" s="277"/>
       <c r="D10" s="217">
         <f>Paėmimas!L10</f>
         <v>0.03</v>
@@ -7044,7 +7044,7 @@
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="54"/>
       <c r="B11" s="21"/>
-      <c r="C11" s="254"/>
+      <c r="C11" s="277"/>
       <c r="D11" s="217">
         <f>Paėmimas!L11</f>
         <v>0.03</v>
@@ -7081,7 +7081,7 @@
     <row r="12" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="54"/>
       <c r="B12" s="21"/>
-      <c r="C12" s="254"/>
+      <c r="C12" s="277"/>
       <c r="D12" s="217">
         <f>Paėmimas!L12</f>
         <v>0.03</v>
@@ -7118,7 +7118,7 @@
     <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="54"/>
       <c r="B13" s="21"/>
-      <c r="C13" s="254"/>
+      <c r="C13" s="277"/>
       <c r="D13" s="217">
         <f>Paėmimas!L13</f>
         <v>0.03</v>
@@ -7155,7 +7155,7 @@
     <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="54"/>
       <c r="B14" s="21"/>
-      <c r="C14" s="254"/>
+      <c r="C14" s="277"/>
       <c r="D14" s="217">
         <f>Paėmimas!L14</f>
         <v>0.03</v>
@@ -7192,7 +7192,7 @@
     <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="54"/>
       <c r="B15" s="21"/>
-      <c r="C15" s="254"/>
+      <c r="C15" s="277"/>
       <c r="D15" s="217">
         <f>Paėmimas!L15</f>
         <v>0.03</v>
@@ -7229,7 +7229,7 @@
     <row r="16" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="54"/>
       <c r="B16" s="21"/>
-      <c r="C16" s="254"/>
+      <c r="C16" s="277"/>
       <c r="D16" s="217">
         <f>Paėmimas!L16</f>
         <v>0.03</v>
@@ -7266,7 +7266,7 @@
     <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="54"/>
       <c r="B17" s="21"/>
-      <c r="C17" s="254"/>
+      <c r="C17" s="277"/>
       <c r="D17" s="217">
         <f>Paėmimas!L17</f>
         <v>0.03</v>
@@ -7303,7 +7303,7 @@
     <row r="18" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="54"/>
       <c r="B18" s="21"/>
-      <c r="C18" s="254"/>
+      <c r="C18" s="277"/>
       <c r="D18" s="217">
         <f>Paėmimas!L18</f>
         <v>0.03</v>
@@ -7340,7 +7340,7 @@
     <row r="19" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="54"/>
       <c r="B19" s="21"/>
-      <c r="C19" s="254"/>
+      <c r="C19" s="277"/>
       <c r="D19" s="217">
         <f>Paėmimas!L19</f>
         <v>0.03</v>
@@ -7377,7 +7377,7 @@
     <row r="20" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="54"/>
       <c r="B20" s="21"/>
-      <c r="C20" s="254"/>
+      <c r="C20" s="277"/>
       <c r="D20" s="217">
         <f>Paėmimas!L20</f>
         <v>0.03</v>
@@ -7414,7 +7414,7 @@
     <row r="21" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="54"/>
       <c r="B21" s="21"/>
-      <c r="C21" s="254"/>
+      <c r="C21" s="277"/>
       <c r="D21" s="217">
         <f>Paėmimas!L21</f>
         <v>0.03</v>
@@ -7451,7 +7451,7 @@
     <row r="22" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="56"/>
       <c r="B22" s="57"/>
-      <c r="C22" s="255"/>
+      <c r="C22" s="278"/>
       <c r="D22" s="217">
         <f>Paėmimas!L22</f>
         <v>0.03</v>
@@ -7582,10 +7582,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="251" t="s">
+      <c r="C1" s="274" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="251"/>
+      <c r="D1" s="274"/>
       <c r="R1" s="16"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -7808,12 +7808,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="251" t="s">
+      <c r="C1" s="274" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="251"/>
-      <c r="E1" s="251"/>
-      <c r="F1" s="251"/>
+      <c r="D1" s="274"/>
+      <c r="E1" s="274"/>
+      <c r="F1" s="274"/>
     </row>
     <row r="2" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="279" t="s">
@@ -8360,6 +8360,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentas" ma:contentTypeID="0x010100BAB57CF81AE55C4698AAD22D302297F0" ma:contentTypeVersion="18" ma:contentTypeDescription="Kurkite naują dokumentą." ma:contentTypeScope="" ma:versionID="49ab401eb4052690d2a2629974c22fd6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="453e7e53-5eb2-45cf-b2ab-34c867e554b8" xmlns:ns3="aa0d983d-359a-438c-9953-3af1a8ac0831" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ab9969d50e0b13c63bc5bd0499c928dc" ns2:_="" ns3:_="">
     <xsd:import namespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
@@ -8614,15 +8623,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
   <ds:schemaRefs>
@@ -8635,6 +8635,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{051C3312-BA73-4284-BC62-F5F884DAFCDD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8651,12 +8659,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Perkeliami Paemimas lapo stulpeliu komplektai
</commit_message>
<xml_diff>
--- a/Ivestis1.xlsx
+++ b/Ivestis1.xlsx
@@ -2630,6 +2630,39 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
@@ -2721,39 +2754,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3258,31 +3258,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="D3" s="249" t="s">
+      <c r="D3" s="258" t="s">
         <v>105</v>
       </c>
-      <c r="E3" s="249"/>
-      <c r="F3" s="249"/>
-      <c r="G3" s="249"/>
-      <c r="H3" s="249"/>
-      <c r="I3" s="249"/>
-      <c r="J3" s="249"/>
-      <c r="K3" s="249"/>
-      <c r="L3" s="249"/>
-      <c r="M3" s="249"/>
-      <c r="N3" s="249"/>
-      <c r="O3" s="249"/>
-      <c r="P3" s="249"/>
-      <c r="Q3" s="249"/>
-      <c r="R3" s="249"/>
-      <c r="S3" s="249"/>
-      <c r="T3" s="249"/>
-      <c r="U3" s="249"/>
-      <c r="V3" s="249"/>
-      <c r="W3" s="249"/>
-      <c r="X3" s="249"/>
-      <c r="Y3" s="249"/>
-      <c r="Z3" s="249"/>
+      <c r="E3" s="258"/>
+      <c r="F3" s="258"/>
+      <c r="G3" s="258"/>
+      <c r="H3" s="258"/>
+      <c r="I3" s="258"/>
+      <c r="J3" s="258"/>
+      <c r="K3" s="258"/>
+      <c r="L3" s="258"/>
+      <c r="M3" s="258"/>
+      <c r="N3" s="258"/>
+      <c r="O3" s="258"/>
+      <c r="P3" s="258"/>
+      <c r="Q3" s="258"/>
+      <c r="R3" s="258"/>
+      <c r="S3" s="258"/>
+      <c r="T3" s="258"/>
+      <c r="U3" s="258"/>
+      <c r="V3" s="258"/>
+      <c r="W3" s="258"/>
+      <c r="X3" s="258"/>
+      <c r="Y3" s="258"/>
+      <c r="Z3" s="258"/>
     </row>
     <row r="5" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
@@ -3371,13 +3371,13 @@
       </c>
     </row>
     <row r="6" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="250">
+      <c r="A6" s="259">
         <v>46210</v>
       </c>
-      <c r="B6" s="253">
+      <c r="B6" s="262">
         <v>7</v>
       </c>
-      <c r="C6" s="254" t="s">
+      <c r="C6" s="263" t="s">
         <v>134</v>
       </c>
       <c r="D6" s="143">
@@ -3463,14 +3463,14 @@
         <f>Aerodinamika!G23</f>
         <v>1.2973599999999998</v>
       </c>
-      <c r="AB6" s="247" t="s">
+      <c r="AB6" s="256" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="251"/>
-      <c r="B7" s="251"/>
-      <c r="C7" s="255"/>
+      <c r="A7" s="260"/>
+      <c r="B7" s="260"/>
+      <c r="C7" s="264"/>
       <c r="D7" s="143">
         <v>2</v>
       </c>
@@ -3550,12 +3550,12 @@
         <f>O6*X7</f>
         <v>0.34775490281286214</v>
       </c>
-      <c r="AB7" s="248"/>
+      <c r="AB7" s="257"/>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="251"/>
-      <c r="B8" s="251"/>
-      <c r="C8" s="255"/>
+      <c r="A8" s="260"/>
+      <c r="B8" s="260"/>
+      <c r="C8" s="264"/>
       <c r="D8" s="166">
         <v>3</v>
       </c>
@@ -3601,9 +3601,9 @@
       <c r="S8" s="142"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A9" s="251"/>
-      <c r="B9" s="251"/>
-      <c r="C9" s="255"/>
+      <c r="A9" s="260"/>
+      <c r="B9" s="260"/>
+      <c r="C9" s="264"/>
       <c r="D9" s="143">
         <v>4</v>
       </c>
@@ -3653,9 +3653,9 @@
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A10" s="251"/>
-      <c r="B10" s="251"/>
-      <c r="C10" s="255"/>
+      <c r="A10" s="260"/>
+      <c r="B10" s="260"/>
+      <c r="C10" s="264"/>
       <c r="D10" s="143">
         <v>5</v>
       </c>
@@ -3694,9 +3694,9 @@
       <c r="N10" s="209"/>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A11" s="251"/>
-      <c r="B11" s="251"/>
-      <c r="C11" s="255"/>
+      <c r="A11" s="260"/>
+      <c r="B11" s="260"/>
+      <c r="C11" s="264"/>
       <c r="D11" s="166">
         <v>6</v>
       </c>
@@ -3735,9 +3735,9 @@
       <c r="N11" s="209"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A12" s="251"/>
-      <c r="B12" s="251"/>
-      <c r="C12" s="255"/>
+      <c r="A12" s="260"/>
+      <c r="B12" s="260"/>
+      <c r="C12" s="264"/>
       <c r="D12" s="143">
         <v>7</v>
       </c>
@@ -3776,9 +3776,9 @@
       <c r="N12" s="209"/>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A13" s="251"/>
-      <c r="B13" s="251"/>
-      <c r="C13" s="255"/>
+      <c r="A13" s="260"/>
+      <c r="B13" s="260"/>
+      <c r="C13" s="264"/>
       <c r="D13" s="143">
         <v>8</v>
       </c>
@@ -3818,9 +3818,9 @@
       <c r="O13" s="137"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A14" s="251"/>
-      <c r="B14" s="251"/>
-      <c r="C14" s="255"/>
+      <c r="A14" s="260"/>
+      <c r="B14" s="260"/>
+      <c r="C14" s="264"/>
       <c r="D14" s="166">
         <v>9</v>
       </c>
@@ -3863,9 +3863,9 @@
       <c r="U14" s="38"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A15" s="251"/>
-      <c r="B15" s="251"/>
-      <c r="C15" s="255"/>
+      <c r="A15" s="260"/>
+      <c r="B15" s="260"/>
+      <c r="C15" s="264"/>
       <c r="D15" s="143">
         <v>10</v>
       </c>
@@ -3908,9 +3908,9 @@
       <c r="U15" s="38"/>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A16" s="251"/>
-      <c r="B16" s="251"/>
-      <c r="C16" s="255"/>
+      <c r="A16" s="260"/>
+      <c r="B16" s="260"/>
+      <c r="C16" s="264"/>
       <c r="D16" s="143">
         <v>11</v>
       </c>
@@ -3953,9 +3953,9 @@
       <c r="U16" s="38"/>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A17" s="251"/>
-      <c r="B17" s="251"/>
-      <c r="C17" s="255"/>
+      <c r="A17" s="260"/>
+      <c r="B17" s="260"/>
+      <c r="C17" s="264"/>
       <c r="D17" s="166">
         <v>12</v>
       </c>
@@ -3998,9 +3998,9 @@
       <c r="U17" s="38"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A18" s="251"/>
-      <c r="B18" s="251"/>
-      <c r="C18" s="255"/>
+      <c r="A18" s="260"/>
+      <c r="B18" s="260"/>
+      <c r="C18" s="264"/>
       <c r="D18" s="143">
         <v>13</v>
       </c>
@@ -4043,9 +4043,9 @@
       <c r="U18" s="38"/>
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A19" s="251"/>
-      <c r="B19" s="251"/>
-      <c r="C19" s="255"/>
+      <c r="A19" s="260"/>
+      <c r="B19" s="260"/>
+      <c r="C19" s="264"/>
       <c r="D19" s="143">
         <v>14</v>
       </c>
@@ -4088,9 +4088,9 @@
       <c r="U19" s="38"/>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A20" s="251"/>
-      <c r="B20" s="251"/>
-      <c r="C20" s="255"/>
+      <c r="A20" s="260"/>
+      <c r="B20" s="260"/>
+      <c r="C20" s="264"/>
       <c r="D20" s="166">
         <v>15</v>
       </c>
@@ -4133,9 +4133,9 @@
       <c r="U20" s="38"/>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A21" s="251"/>
-      <c r="B21" s="251"/>
-      <c r="C21" s="255"/>
+      <c r="A21" s="260"/>
+      <c r="B21" s="260"/>
+      <c r="C21" s="264"/>
       <c r="D21" s="143">
         <v>16</v>
       </c>
@@ -4178,9 +4178,9 @@
       <c r="U21" s="38"/>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A22" s="252"/>
-      <c r="B22" s="252"/>
-      <c r="C22" s="256"/>
+      <c r="A22" s="261"/>
+      <c r="B22" s="261"/>
+      <c r="C22" s="265"/>
       <c r="D22" s="143">
         <v>17</v>
       </c>
@@ -4284,11 +4284,11 @@
         <v>0</v>
       </c>
       <c r="N24" s="71"/>
-      <c r="O24" s="257" t="s">
+      <c r="O24" s="266" t="s">
         <v>131</v>
       </c>
-      <c r="P24" s="258"/>
-      <c r="Q24" s="258"/>
+      <c r="P24" s="267"/>
+      <c r="Q24" s="267"/>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="177"/>
@@ -4323,30 +4323,30 @@
       <c r="A28" s="177"/>
       <c r="B28" s="177"/>
       <c r="C28" s="177"/>
-      <c r="D28" s="259" t="s">
+      <c r="D28" s="268" t="s">
         <v>133</v>
       </c>
-      <c r="E28" s="249"/>
-      <c r="F28" s="249"/>
-      <c r="G28" s="249"/>
-      <c r="H28" s="249"/>
-      <c r="I28" s="249"/>
-      <c r="J28" s="249"/>
-      <c r="K28" s="249"/>
-      <c r="L28" s="249"/>
-      <c r="M28" s="249"/>
-      <c r="N28" s="249"/>
-      <c r="O28" s="249"/>
-      <c r="P28" s="249"/>
-      <c r="Q28" s="249"/>
-      <c r="R28" s="249"/>
-      <c r="S28" s="249"/>
-      <c r="T28" s="249"/>
-      <c r="U28" s="249"/>
-      <c r="V28" s="249"/>
-      <c r="W28" s="249"/>
-      <c r="X28" s="249"/>
-      <c r="Y28" s="249"/>
+      <c r="E28" s="258"/>
+      <c r="F28" s="258"/>
+      <c r="G28" s="258"/>
+      <c r="H28" s="258"/>
+      <c r="I28" s="258"/>
+      <c r="J28" s="258"/>
+      <c r="K28" s="258"/>
+      <c r="L28" s="258"/>
+      <c r="M28" s="258"/>
+      <c r="N28" s="258"/>
+      <c r="O28" s="258"/>
+      <c r="P28" s="258"/>
+      <c r="Q28" s="258"/>
+      <c r="R28" s="258"/>
+      <c r="S28" s="258"/>
+      <c r="T28" s="258"/>
+      <c r="U28" s="258"/>
+      <c r="V28" s="258"/>
+      <c r="W28" s="258"/>
+      <c r="X28" s="258"/>
+      <c r="Y28" s="258"/>
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="177"/>
@@ -4451,9 +4451,9 @@
       </c>
     </row>
     <row r="31" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="260"/>
-      <c r="B31" s="260"/>
-      <c r="C31" s="260"/>
+      <c r="A31" s="269"/>
+      <c r="B31" s="269"/>
+      <c r="C31" s="269"/>
       <c r="D31" s="143">
         <v>5</v>
       </c>
@@ -4528,12 +4528,12 @@
       <c r="AA31" s="187">
         <v>1.29</v>
       </c>
-      <c r="AB31" s="247"/>
+      <c r="AB31" s="256"/>
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A32" s="261"/>
-      <c r="B32" s="261"/>
-      <c r="C32" s="261"/>
+      <c r="A32" s="270"/>
+      <c r="B32" s="270"/>
+      <c r="C32" s="270"/>
       <c r="D32" s="143">
         <v>14</v>
       </c>
@@ -4602,12 +4602,12 @@
         <f>O31*X32</f>
         <v>0.90295018924227777</v>
       </c>
-      <c r="AB32" s="248"/>
+      <c r="AB32" s="257"/>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A33" s="261"/>
-      <c r="B33" s="261"/>
-      <c r="C33" s="261"/>
+      <c r="A33" s="270"/>
+      <c r="B33" s="270"/>
+      <c r="C33" s="270"/>
       <c r="D33" s="166">
         <v>24</v>
       </c>
@@ -4644,9 +4644,9 @@
       <c r="S33" s="142"/>
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A34" s="261"/>
-      <c r="B34" s="261"/>
-      <c r="C34" s="261"/>
+      <c r="A34" s="270"/>
+      <c r="B34" s="270"/>
+      <c r="C34" s="270"/>
       <c r="D34" s="143">
         <v>33</v>
       </c>
@@ -4687,9 +4687,9 @@
       </c>
     </row>
     <row r="35" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A35" s="261"/>
-      <c r="B35" s="261"/>
-      <c r="C35" s="261"/>
+      <c r="A35" s="270"/>
+      <c r="B35" s="270"/>
+      <c r="C35" s="270"/>
       <c r="D35" s="143">
         <v>42</v>
       </c>
@@ -4719,9 +4719,9 @@
       <c r="N35" s="149"/>
     </row>
     <row r="36" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A36" s="261"/>
-      <c r="B36" s="261"/>
-      <c r="C36" s="261"/>
+      <c r="A36" s="270"/>
+      <c r="B36" s="270"/>
+      <c r="C36" s="270"/>
       <c r="D36" s="143">
         <v>52</v>
       </c>
@@ -4751,9 +4751,9 @@
       <c r="N36" s="149"/>
     </row>
     <row r="37" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A37" s="261"/>
-      <c r="B37" s="261"/>
-      <c r="C37" s="261"/>
+      <c r="A37" s="270"/>
+      <c r="B37" s="270"/>
+      <c r="C37" s="270"/>
       <c r="D37" s="143">
         <v>61</v>
       </c>
@@ -4783,9 +4783,9 @@
       <c r="N37" s="149"/>
     </row>
     <row r="38" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A38" s="261"/>
-      <c r="B38" s="261"/>
-      <c r="C38" s="261"/>
+      <c r="A38" s="270"/>
+      <c r="B38" s="270"/>
+      <c r="C38" s="270"/>
       <c r="D38" s="143">
         <v>71</v>
       </c>
@@ -4816,9 +4816,9 @@
       <c r="O38" s="137"/>
     </row>
     <row r="39" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A39" s="261"/>
-      <c r="B39" s="261"/>
-      <c r="C39" s="261"/>
+      <c r="A39" s="270"/>
+      <c r="B39" s="270"/>
+      <c r="C39" s="270"/>
       <c r="D39" s="143">
         <v>80</v>
       </c>
@@ -4852,9 +4852,9 @@
       <c r="U39" s="38"/>
     </row>
     <row r="40" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A40" s="261"/>
-      <c r="B40" s="261"/>
-      <c r="C40" s="261"/>
+      <c r="A40" s="270"/>
+      <c r="B40" s="270"/>
+      <c r="C40" s="270"/>
       <c r="D40" s="143">
         <v>89</v>
       </c>
@@ -4884,9 +4884,9 @@
       <c r="N40" s="143"/>
     </row>
     <row r="41" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A41" s="261"/>
-      <c r="B41" s="261"/>
-      <c r="C41" s="261"/>
+      <c r="A41" s="270"/>
+      <c r="B41" s="270"/>
+      <c r="C41" s="270"/>
       <c r="D41" s="143">
         <v>99</v>
       </c>
@@ -4916,9 +4916,9 @@
       <c r="N41" s="143"/>
     </row>
     <row r="42" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A42" s="261"/>
-      <c r="B42" s="261"/>
-      <c r="C42" s="261"/>
+      <c r="A42" s="270"/>
+      <c r="B42" s="270"/>
+      <c r="C42" s="270"/>
       <c r="D42" s="143">
         <v>108</v>
       </c>
@@ -4948,9 +4948,9 @@
       <c r="N42" s="143"/>
     </row>
     <row r="43" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A43" s="261"/>
-      <c r="B43" s="261"/>
-      <c r="C43" s="261"/>
+      <c r="A43" s="270"/>
+      <c r="B43" s="270"/>
+      <c r="C43" s="270"/>
       <c r="D43" s="143">
         <v>118</v>
       </c>
@@ -4980,9 +4980,9 @@
       <c r="N43" s="143"/>
     </row>
     <row r="44" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A44" s="261"/>
-      <c r="B44" s="261"/>
-      <c r="C44" s="261"/>
+      <c r="A44" s="270"/>
+      <c r="B44" s="270"/>
+      <c r="C44" s="270"/>
       <c r="D44" s="143">
         <v>127</v>
       </c>
@@ -5012,9 +5012,9 @@
       <c r="N44" s="143"/>
     </row>
     <row r="45" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A45" s="261"/>
-      <c r="B45" s="261"/>
-      <c r="C45" s="261"/>
+      <c r="A45" s="270"/>
+      <c r="B45" s="270"/>
+      <c r="C45" s="270"/>
       <c r="D45" s="143">
         <v>136</v>
       </c>
@@ -5044,9 +5044,9 @@
       <c r="N45" s="143"/>
     </row>
     <row r="46" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A46" s="261"/>
-      <c r="B46" s="261"/>
-      <c r="C46" s="261"/>
+      <c r="A46" s="270"/>
+      <c r="B46" s="270"/>
+      <c r="C46" s="270"/>
       <c r="D46" s="143">
         <v>146</v>
       </c>
@@ -5076,9 +5076,9 @@
       <c r="N46" s="143"/>
     </row>
     <row r="47" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A47" s="262"/>
-      <c r="B47" s="262"/>
-      <c r="C47" s="262"/>
+      <c r="A47" s="271"/>
+      <c r="B47" s="271"/>
+      <c r="C47" s="271"/>
       <c r="D47" s="143">
         <v>155</v>
       </c>
@@ -5167,18 +5167,18 @@
       <c r="I2" s="10"/>
     </row>
     <row r="3" spans="1:12" ht="15" x14ac:dyDescent="0.3">
-      <c r="A3" s="263" t="s">
+      <c r="A3" s="272" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="263"/>
-      <c r="C3" s="263"/>
-      <c r="D3" s="263"/>
-      <c r="E3" s="263"/>
-      <c r="F3" s="263"/>
-      <c r="G3" s="263"/>
-      <c r="H3" s="263"/>
-      <c r="I3" s="263"/>
-      <c r="J3" s="263"/>
+      <c r="B3" s="272"/>
+      <c r="C3" s="272"/>
+      <c r="D3" s="272"/>
+      <c r="E3" s="272"/>
+      <c r="F3" s="272"/>
+      <c r="G3" s="272"/>
+      <c r="H3" s="272"/>
+      <c r="I3" s="272"/>
+      <c r="J3" s="272"/>
     </row>
     <row r="4" spans="1:12" ht="14" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
@@ -5325,46 +5325,46 @@
       <c r="L10" s="45"/>
     </row>
     <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H11" s="264" t="s">
+      <c r="H11" s="273" t="s">
         <v>29</v>
       </c>
-      <c r="I11" s="267" t="s">
+      <c r="I11" s="276" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H12" s="265"/>
-      <c r="I12" s="268"/>
+      <c r="H12" s="274"/>
+      <c r="I12" s="277"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H13" s="265"/>
-      <c r="I13" s="268"/>
+      <c r="H13" s="274"/>
+      <c r="I13" s="277"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H14" s="265"/>
-      <c r="I14" s="268"/>
+      <c r="H14" s="274"/>
+      <c r="I14" s="277"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H15" s="265"/>
-      <c r="I15" s="268"/>
+      <c r="H15" s="274"/>
+      <c r="I15" s="277"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H16" s="265"/>
-      <c r="I16" s="268"/>
+      <c r="H16" s="274"/>
+      <c r="I16" s="277"/>
     </row>
     <row r="17" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H17" s="265"/>
-      <c r="I17" s="268"/>
+      <c r="H17" s="274"/>
+      <c r="I17" s="277"/>
     </row>
     <row r="18" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H18" s="266"/>
-      <c r="I18" s="268"/>
+      <c r="H18" s="275"/>
+      <c r="I18" s="277"/>
     </row>
     <row r="19" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="I19" s="268"/>
+      <c r="I19" s="277"/>
     </row>
     <row r="20" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="I20" s="269"/>
+      <c r="I20" s="278"/>
     </row>
     <row r="23" spans="8:9" ht="14" x14ac:dyDescent="0.3">
       <c r="I23" s="52"/>
@@ -5425,35 +5425,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="274" t="s">
+      <c r="C1" s="251" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="274"/>
+      <c r="D1" s="251"/>
       <c r="E1" s="15"/>
       <c r="S1" s="80"/>
     </row>
     <row r="2" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="275" t="s">
+      <c r="A2" s="252" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="275"/>
-      <c r="C2" s="275"/>
-      <c r="D2" s="275"/>
-      <c r="E2" s="275"/>
-      <c r="F2" s="275"/>
-      <c r="G2" s="275"/>
-      <c r="H2" s="275"/>
-      <c r="I2" s="275"/>
-      <c r="J2" s="275"/>
-      <c r="K2" s="275"/>
-      <c r="L2" s="275"/>
-      <c r="M2" s="275"/>
-      <c r="N2" s="275"/>
-      <c r="O2" s="275"/>
-      <c r="P2" s="275"/>
-      <c r="Q2" s="275"/>
-      <c r="R2" s="275"/>
-      <c r="S2" s="275"/>
+      <c r="B2" s="252"/>
+      <c r="C2" s="252"/>
+      <c r="D2" s="252"/>
+      <c r="E2" s="252"/>
+      <c r="F2" s="252"/>
+      <c r="G2" s="252"/>
+      <c r="H2" s="252"/>
+      <c r="I2" s="252"/>
+      <c r="J2" s="252"/>
+      <c r="K2" s="252"/>
+      <c r="L2" s="252"/>
+      <c r="M2" s="252"/>
+      <c r="N2" s="252"/>
+      <c r="O2" s="252"/>
+      <c r="P2" s="252"/>
+      <c r="Q2" s="252"/>
+      <c r="R2" s="252"/>
+      <c r="S2" s="252"/>
     </row>
     <row r="3" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="81"/>
@@ -5562,7 +5562,7 @@
       <c r="B6" s="49">
         <v>1</v>
       </c>
-      <c r="C6" s="276" t="str">
+      <c r="C6" s="253" t="str">
         <f>Greitis!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -5642,7 +5642,7 @@
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="36"/>
       <c r="B7" s="33"/>
-      <c r="C7" s="277"/>
+      <c r="C7" s="254"/>
       <c r="D7" s="17"/>
       <c r="E7" s="18"/>
       <c r="F7" s="211">
@@ -5713,7 +5713,7 @@
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" s="36"/>
       <c r="B8" s="33"/>
-      <c r="C8" s="277"/>
+      <c r="C8" s="254"/>
       <c r="D8" s="17"/>
       <c r="E8" s="18"/>
       <c r="F8" s="211">
@@ -5784,7 +5784,7 @@
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="36"/>
       <c r="B9" s="33"/>
-      <c r="C9" s="277"/>
+      <c r="C9" s="254"/>
       <c r="D9" s="85"/>
       <c r="E9" s="85"/>
       <c r="F9" s="211">
@@ -5858,7 +5858,7 @@
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="85"/>
       <c r="B10" s="85"/>
-      <c r="C10" s="277"/>
+      <c r="C10" s="254"/>
       <c r="D10" s="85"/>
       <c r="E10" s="85"/>
       <c r="F10" s="211">
@@ -5908,13 +5908,13 @@
       </c>
       <c r="R10" s="85"/>
       <c r="S10" s="85"/>
-      <c r="T10" s="271" t="s">
+      <c r="T10" s="248" t="s">
         <v>31</v>
       </c>
-      <c r="U10" s="271" t="s">
+      <c r="U10" s="248" t="s">
         <v>32</v>
       </c>
-      <c r="V10" s="270" t="s">
+      <c r="V10" s="247" t="s">
         <v>36</v>
       </c>
       <c r="X10" s="205">
@@ -5929,7 +5929,7 @@
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="85"/>
       <c r="B11" s="85"/>
-      <c r="C11" s="277"/>
+      <c r="C11" s="254"/>
       <c r="D11" s="85"/>
       <c r="E11" s="85"/>
       <c r="F11" s="211">
@@ -5979,9 +5979,9 @@
       </c>
       <c r="R11" s="85"/>
       <c r="S11" s="85"/>
-      <c r="T11" s="272"/>
-      <c r="U11" s="272"/>
-      <c r="V11" s="270"/>
+      <c r="T11" s="249"/>
+      <c r="U11" s="249"/>
+      <c r="V11" s="247"/>
       <c r="X11" s="205">
         <f>Greitis!E11</f>
         <v>0.14000000000000001</v>
@@ -5994,7 +5994,7 @@
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="85"/>
       <c r="B12" s="85"/>
-      <c r="C12" s="277"/>
+      <c r="C12" s="254"/>
       <c r="D12" s="85"/>
       <c r="E12" s="85"/>
       <c r="F12" s="211">
@@ -6044,9 +6044,9 @@
       </c>
       <c r="R12" s="85"/>
       <c r="S12" s="85"/>
-      <c r="T12" s="273"/>
-      <c r="U12" s="273"/>
-      <c r="V12" s="270"/>
+      <c r="T12" s="250"/>
+      <c r="U12" s="250"/>
+      <c r="V12" s="247"/>
       <c r="X12" s="205">
         <f>Greitis!E12</f>
         <v>0.14000000000000001</v>
@@ -6059,7 +6059,7 @@
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="85"/>
       <c r="B13" s="85"/>
-      <c r="C13" s="277"/>
+      <c r="C13" s="254"/>
       <c r="D13" s="85"/>
       <c r="E13" s="85"/>
       <c r="F13" s="211">
@@ -6121,7 +6121,7 @@
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="85"/>
       <c r="B14" s="85"/>
-      <c r="C14" s="277"/>
+      <c r="C14" s="254"/>
       <c r="D14" s="85"/>
       <c r="E14" s="85"/>
       <c r="F14" s="211">
@@ -6183,7 +6183,7 @@
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="85"/>
       <c r="B15" s="85"/>
-      <c r="C15" s="277"/>
+      <c r="C15" s="254"/>
       <c r="D15" s="85"/>
       <c r="E15" s="85"/>
       <c r="F15" s="211">
@@ -6245,7 +6245,7 @@
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="85"/>
       <c r="B16" s="85"/>
-      <c r="C16" s="277"/>
+      <c r="C16" s="254"/>
       <c r="D16" s="85"/>
       <c r="E16" s="85"/>
       <c r="F16" s="211">
@@ -6307,7 +6307,7 @@
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" s="85"/>
       <c r="B17" s="85"/>
-      <c r="C17" s="277"/>
+      <c r="C17" s="254"/>
       <c r="D17" s="85"/>
       <c r="E17" s="85"/>
       <c r="F17" s="211">
@@ -6369,7 +6369,7 @@
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" s="85"/>
       <c r="B18" s="85"/>
-      <c r="C18" s="277"/>
+      <c r="C18" s="254"/>
       <c r="D18" s="85"/>
       <c r="E18" s="85"/>
       <c r="F18" s="211">
@@ -6431,7 +6431,7 @@
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" s="85"/>
       <c r="B19" s="85"/>
-      <c r="C19" s="277"/>
+      <c r="C19" s="254"/>
       <c r="D19" s="85"/>
       <c r="E19" s="85"/>
       <c r="F19" s="211">
@@ -6493,7 +6493,7 @@
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" s="85"/>
       <c r="B20" s="85"/>
-      <c r="C20" s="277"/>
+      <c r="C20" s="254"/>
       <c r="D20" s="85"/>
       <c r="E20" s="85"/>
       <c r="F20" s="211">
@@ -6555,7 +6555,7 @@
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" s="85"/>
       <c r="B21" s="85"/>
-      <c r="C21" s="277"/>
+      <c r="C21" s="254"/>
       <c r="D21" s="85"/>
       <c r="E21" s="85"/>
       <c r="F21" s="211">
@@ -6617,7 +6617,7 @@
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" s="86"/>
       <c r="B22" s="86"/>
-      <c r="C22" s="278"/>
+      <c r="C22" s="255"/>
       <c r="D22" s="86"/>
       <c r="E22" s="86"/>
       <c r="F22" s="211">
@@ -6763,10 +6763,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="274" t="s">
+      <c r="C1" s="251" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="274"/>
+      <c r="D1" s="251"/>
       <c r="Q1" s="16"/>
     </row>
     <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -6844,7 +6844,7 @@
         <f>Paėmimas!B6</f>
         <v>1</v>
       </c>
-      <c r="C6" s="276" t="str">
+      <c r="C6" s="253" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -6896,7 +6896,7 @@
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="54"/>
       <c r="B7" s="21"/>
-      <c r="C7" s="277"/>
+      <c r="C7" s="254"/>
       <c r="D7" s="217">
         <f>Paėmimas!L7</f>
         <v>0.03</v>
@@ -6933,7 +6933,7 @@
     <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="54"/>
       <c r="B8" s="21"/>
-      <c r="C8" s="277"/>
+      <c r="C8" s="254"/>
       <c r="D8" s="217">
         <f>Paėmimas!L8</f>
         <v>0.03</v>
@@ -6970,7 +6970,7 @@
     <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="54"/>
       <c r="B9" s="21"/>
-      <c r="C9" s="277"/>
+      <c r="C9" s="254"/>
       <c r="D9" s="217">
         <f>Paėmimas!L9</f>
         <v>0.03</v>
@@ -7007,7 +7007,7 @@
     <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="54"/>
       <c r="B10" s="21"/>
-      <c r="C10" s="277"/>
+      <c r="C10" s="254"/>
       <c r="D10" s="217">
         <f>Paėmimas!L10</f>
         <v>0.03</v>
@@ -7044,7 +7044,7 @@
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="54"/>
       <c r="B11" s="21"/>
-      <c r="C11" s="277"/>
+      <c r="C11" s="254"/>
       <c r="D11" s="217">
         <f>Paėmimas!L11</f>
         <v>0.03</v>
@@ -7081,7 +7081,7 @@
     <row r="12" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="54"/>
       <c r="B12" s="21"/>
-      <c r="C12" s="277"/>
+      <c r="C12" s="254"/>
       <c r="D12" s="217">
         <f>Paėmimas!L12</f>
         <v>0.03</v>
@@ -7118,7 +7118,7 @@
     <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="54"/>
       <c r="B13" s="21"/>
-      <c r="C13" s="277"/>
+      <c r="C13" s="254"/>
       <c r="D13" s="217">
         <f>Paėmimas!L13</f>
         <v>0.03</v>
@@ -7155,7 +7155,7 @@
     <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="54"/>
       <c r="B14" s="21"/>
-      <c r="C14" s="277"/>
+      <c r="C14" s="254"/>
       <c r="D14" s="217">
         <f>Paėmimas!L14</f>
         <v>0.03</v>
@@ -7192,7 +7192,7 @@
     <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="54"/>
       <c r="B15" s="21"/>
-      <c r="C15" s="277"/>
+      <c r="C15" s="254"/>
       <c r="D15" s="217">
         <f>Paėmimas!L15</f>
         <v>0.03</v>
@@ -7229,7 +7229,7 @@
     <row r="16" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="54"/>
       <c r="B16" s="21"/>
-      <c r="C16" s="277"/>
+      <c r="C16" s="254"/>
       <c r="D16" s="217">
         <f>Paėmimas!L16</f>
         <v>0.03</v>
@@ -7266,7 +7266,7 @@
     <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="54"/>
       <c r="B17" s="21"/>
-      <c r="C17" s="277"/>
+      <c r="C17" s="254"/>
       <c r="D17" s="217">
         <f>Paėmimas!L17</f>
         <v>0.03</v>
@@ -7303,7 +7303,7 @@
     <row r="18" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="54"/>
       <c r="B18" s="21"/>
-      <c r="C18" s="277"/>
+      <c r="C18" s="254"/>
       <c r="D18" s="217">
         <f>Paėmimas!L18</f>
         <v>0.03</v>
@@ -7340,7 +7340,7 @@
     <row r="19" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="54"/>
       <c r="B19" s="21"/>
-      <c r="C19" s="277"/>
+      <c r="C19" s="254"/>
       <c r="D19" s="217">
         <f>Paėmimas!L19</f>
         <v>0.03</v>
@@ -7377,7 +7377,7 @@
     <row r="20" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="54"/>
       <c r="B20" s="21"/>
-      <c r="C20" s="277"/>
+      <c r="C20" s="254"/>
       <c r="D20" s="217">
         <f>Paėmimas!L20</f>
         <v>0.03</v>
@@ -7414,7 +7414,7 @@
     <row r="21" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="54"/>
       <c r="B21" s="21"/>
-      <c r="C21" s="277"/>
+      <c r="C21" s="254"/>
       <c r="D21" s="217">
         <f>Paėmimas!L21</f>
         <v>0.03</v>
@@ -7451,7 +7451,7 @@
     <row r="22" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="56"/>
       <c r="B22" s="57"/>
-      <c r="C22" s="278"/>
+      <c r="C22" s="255"/>
       <c r="D22" s="217">
         <f>Paėmimas!L22</f>
         <v>0.03</v>
@@ -7582,10 +7582,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="274" t="s">
+      <c r="C1" s="251" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="274"/>
+      <c r="D1" s="251"/>
       <c r="R1" s="16"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -7808,12 +7808,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="274" t="s">
+      <c r="C1" s="251" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="274"/>
-      <c r="E1" s="274"/>
-      <c r="F1" s="274"/>
+      <c r="D1" s="251"/>
+      <c r="E1" s="251"/>
+      <c r="F1" s="251"/>
     </row>
     <row r="2" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="279" t="s">
@@ -8349,26 +8349,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentas" ma:contentTypeID="0x010100BAB57CF81AE55C4698AAD22D302297F0" ma:contentTypeVersion="18" ma:contentTypeDescription="Kurkite naują dokumentą." ma:contentTypeScope="" ma:versionID="49ab401eb4052690d2a2629974c22fd6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="453e7e53-5eb2-45cf-b2ab-34c867e554b8" xmlns:ns3="aa0d983d-359a-438c-9953-3af1a8ac0831" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ab9969d50e0b13c63bc5bd0499c928dc" ns2:_="" ns3:_="">
     <xsd:import namespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
@@ -8623,26 +8603,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
-    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{051C3312-BA73-4284-BC62-F5F884DAFCDD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8659,4 +8640,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>